<commit_message>
docs(fp-183): correct reproducible TCO baseline
</commit_message>
<xml_diff>
--- a/FP-48 TINV02/TINV_Matriz_de_Fuentes_FP-126_actualizada_2026-09-15.xlsx
+++ b/FP-48 TINV02/TINV_Matriz_de_Fuentes_FP-126_actualizada_2026-09-15.xlsx
@@ -2,14 +2,14 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pilares e instrucciones" sheetId="1" r:id="R6b03467af85446f9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Matriz de Fuentes" sheetId="2" r:id="Ref34ddd0c4d24d3b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tablero" sheetId="3" r:id="Ra6b43875244b4b21"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Busquedas ejecutadas" sheetId="4" r:id="R4182998738634ce0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Matriz de precios" sheetId="5" r:id="R89a975d6989c485c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Alternativas" sheetId="6" r:id="Rae410fccf4214b79"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Descartes" sheetId="7" r:id="R8797abfeadd249ea"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Control FP-126" sheetId="8" r:id="Rb3b7d1e5a21f44d5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pilares e instrucciones" sheetId="1" r:id="R742c168b69bf4a82"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Matriz de Fuentes" sheetId="2" r:id="R5d0835b92b5c474b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tablero" sheetId="3" r:id="Racff5ed658444a62"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Busquedas ejecutadas" sheetId="4" r:id="R6e259117163a4cfc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Matriz de precios" sheetId="5" r:id="R3e42ec74cdbd45e2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Alternativas" sheetId="6" r:id="R11473ff5a1674868"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Descartes" sheetId="7" r:id="R336f5abe561b44ff"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Control FP-126" sheetId="8" r:id="R29e2b39709194df6"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1179,9 +1179,6 @@
   </x:si>
   <x:si>
     <x:t xml:space="preserve">FP-126</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Dependencia pendiente</x:t>
   </x:si>
   <x:si>
     <x:t xml:space="preserve">La matriz incluye seis precios Azure verificables y condiciones de cotizacion, pero debe actualizarse cuando FP-51/FP-52 definan la arquitectura y el TCO.</x:t>
@@ -2331,7 +2328,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="1" applyAlignment="1"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="84">
+  <x:cellXfs count="86">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <x:alignment vertical="bottom" wrapText="0"/>
     </x:xf>
@@ -2572,6 +2569,12 @@
       <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="21" fillId="12" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
@@ -7235,349 +7238,814 @@
       </x:c>
     </x:row>
     <x:row r="45" ht="15" customHeight="1">
-      <x:c r="A45" s="22" t="str">
-        <x:f t="shared" ref="A45:A110" si="3">IF(F45="","",TEXT(ROW()-4-1,"000"))</x:f>
-      </x:c>
-      <x:c r="B45" s="10"/>
-      <x:c r="C45" s="10"/>
-      <x:c r="D45" s="10"/>
-      <x:c r="E45" s="10"/>
-      <x:c r="F45" s="10"/>
-      <x:c r="G45" s="10"/>
-      <x:c r="H45" s="10"/>
-      <x:c r="I45" s="10"/>
-      <x:c r="J45" s="10"/>
-      <x:c r="K45" s="10"/>
-      <x:c r="L45" s="10"/>
-      <x:c r="M45" s="22" t="str">
+      <x:c r="A45" s="84" t="str">
+        <x:f t="shared" ref="A45:A110" si="3">IF(F45="","",TEXT(ROW()-5,"000"))</x:f>
+        <x:v>040</x:v>
+      </x:c>
+      <x:c r="B45" s="85" t="str">
+        <x:v>Sitio oficial</x:v>
+      </x:c>
+      <x:c r="C45" s="85" t="str">
+        <x:v>rightsizing, apagado y reducción de desperdicio</x:v>
+      </x:c>
+      <x:c r="D45" s="85" t="n">
+        <x:v>2026</x:v>
+      </x:c>
+      <x:c r="E45" s="85" t="str">
+        <x:v>FinOps Foundation</x:v>
+      </x:c>
+      <x:c r="F45" s="85" t="str">
+        <x:v>Optimize Cloud Usage</x:v>
+      </x:c>
+      <x:c r="G45" s="85" t="str">
+        <x:v>Documentación oficial usada en FP-172 para rightsizing, apagado y reducción de desperdicio.</x:v>
+      </x:c>
+      <x:c r="H45" s="85" t="str">
+        <x:v>rightsizing, apagado y reducción de desperdicio</x:v>
+      </x:c>
+      <x:c r="I45" s="85" t="str">
+        <x:v>https://www.finops.org/framework/capabilities/optimize-cloud-usage/</x:v>
+      </x:c>
+      <x:c r="J45" s="85" t="str">
+        <x:v>Comercial/proveedor</x:v>
+      </x:c>
+      <x:c r="K45" s="85" t="str">
+        <x:v>P2</x:v>
+      </x:c>
+      <x:c r="L45" s="85" t="str">
+        <x:v>5. Caso práctico</x:v>
+      </x:c>
+      <x:c r="M45" s="84" t="str">
         <x:f t="shared" ref="M45:M110" si="4">IF(I45="","",IF(COUNTIFS($I$6:$I$110,I45)&gt;1,IF(COUNTIFS($I$6:$I$110,I45,$K$6:$K$110,"&lt;&gt;"&amp;K45)&gt;0,"SOLAPAMIENTO: otro pilar","Duplicada en el mismo pilar"),""))</x:f>
       </x:c>
-      <x:c r="N45" s="10"/>
-      <x:c r="O45" s="10"/>
-      <x:c r="P45" s="10"/>
-      <x:c r="Q45" s="10"/>
+      <x:c r="N45" s="85" t="str">
+        <x:v>Equipo TINV-04</x:v>
+      </x:c>
+      <x:c r="O45" s="85" t="str">
+        <x:v>Verificada para matriz</x:v>
+      </x:c>
+      <x:c r="P45" s="85" t="str">
+        <x:v>Autoridad: fuente oficial. Uso: rightsizing, apagado y reducción de desperdicio. Límite: validar vigencia, región, SKU y contrato antes de reutilizar cifras. Consultada el 2026-09-16.</x:v>
+      </x:c>
+      <x:c r="Q45" s="85" t="str">
+        <x:v>No</x:v>
+      </x:c>
     </x:row>
     <x:row r="46" ht="15" customHeight="1">
-      <x:c r="A46" s="22" t="str">
-        <x:f t="shared" si="3"/>
-      </x:c>
-      <x:c r="B46" s="10"/>
-      <x:c r="C46" s="10"/>
-      <x:c r="D46" s="10"/>
-      <x:c r="E46" s="10"/>
-      <x:c r="F46" s="10"/>
-      <x:c r="G46" s="10"/>
-      <x:c r="H46" s="10"/>
-      <x:c r="I46" s="10"/>
-      <x:c r="J46" s="10"/>
-      <x:c r="K46" s="10"/>
-      <x:c r="L46" s="10"/>
-      <x:c r="M46" s="22" t="str">
-        <x:f t="shared" si="4"/>
-      </x:c>
-      <x:c r="N46" s="10"/>
-      <x:c r="O46" s="10"/>
-      <x:c r="P46" s="10"/>
-      <x:c r="Q46" s="10"/>
+      <x:c r="A46" s="84" t="str">
+        <x:f t="shared" si="3">IF(F46="","",TEXT(ROW()-5,"000"))</x:f>
+        <x:v>041</x:v>
+      </x:c>
+      <x:c r="B46" s="85" t="str">
+        <x:v>Sitio oficial</x:v>
+      </x:c>
+      <x:c r="C46" s="85" t="str">
+        <x:v>automatización de apagado</x:v>
+      </x:c>
+      <x:c r="D46" s="85" t="n">
+        <x:v>2026</x:v>
+      </x:c>
+      <x:c r="E46" s="85" t="str">
+        <x:v>Microsoft</x:v>
+      </x:c>
+      <x:c r="F46" s="85" t="str">
+        <x:v>Start/stop VMs during off-hours</x:v>
+      </x:c>
+      <x:c r="G46" s="85" t="str">
+        <x:v>Documentación oficial usada en FP-172 para automatización de apagado.</x:v>
+      </x:c>
+      <x:c r="H46" s="85" t="str">
+        <x:v>automatización de apagado</x:v>
+      </x:c>
+      <x:c r="I46" s="85" t="str">
+        <x:v>https://learn.microsoft.com/en-us/azure/automation/automation-solution-vm-management</x:v>
+      </x:c>
+      <x:c r="J46" s="85" t="str">
+        <x:v>Comercial/proveedor</x:v>
+      </x:c>
+      <x:c r="K46" s="85" t="str">
+        <x:v>P2</x:v>
+      </x:c>
+      <x:c r="L46" s="85" t="str">
+        <x:v>5. Caso práctico</x:v>
+      </x:c>
+      <x:c r="M46" s="84" t="str">
+        <x:f t="shared" si="4">IF(I46="","",IF(COUNTIFS($I$6:$I$110,I46)&gt;1,IF(COUNTIFS($I$6:$I$110,I46,$K$6:$K$110,"&lt;&gt;"&amp;K46)&gt;0,"SOLAPAMIENTO: otro pilar","Duplicada en el mismo pilar"),""))</x:f>
+      </x:c>
+      <x:c r="N46" s="85" t="str">
+        <x:v>Equipo TINV-04</x:v>
+      </x:c>
+      <x:c r="O46" s="85" t="str">
+        <x:v>Verificada para matriz</x:v>
+      </x:c>
+      <x:c r="P46" s="85" t="str">
+        <x:v>Autoridad: fuente oficial. Uso: automatización de apagado. Límite: validar vigencia, región, SKU y contrato antes de reutilizar cifras. Consultada el 2026-09-16.</x:v>
+      </x:c>
+      <x:c r="Q46" s="85" t="str">
+        <x:v>No</x:v>
+      </x:c>
     </x:row>
     <x:row r="47" ht="15" customHeight="1">
-      <x:c r="A47" s="22" t="str">
-        <x:f t="shared" si="3"/>
-      </x:c>
-      <x:c r="B47" s="10"/>
-      <x:c r="C47" s="10"/>
-      <x:c r="D47" s="10"/>
-      <x:c r="E47" s="10"/>
-      <x:c r="F47" s="10"/>
-      <x:c r="G47" s="10"/>
-      <x:c r="H47" s="10"/>
-      <x:c r="I47" s="10"/>
-      <x:c r="J47" s="10"/>
-      <x:c r="K47" s="10"/>
-      <x:c r="L47" s="10"/>
-      <x:c r="M47" s="22" t="str">
-        <x:f t="shared" si="4"/>
-      </x:c>
-      <x:c r="N47" s="10"/>
-      <x:c r="O47" s="10"/>
-      <x:c r="P47" s="10"/>
-      <x:c r="Q47" s="10"/>
+      <x:c r="A47" s="84" t="str">
+        <x:f t="shared" si="3">IF(F47="","",TEXT(ROW()-5,"000"))</x:f>
+        <x:v>042</x:v>
+      </x:c>
+      <x:c r="B47" s="85" t="str">
+        <x:v>Sitio oficial</x:v>
+      </x:c>
+      <x:c r="C47" s="85" t="str">
+        <x:v>compromisos y cobertura</x:v>
+      </x:c>
+      <x:c r="D47" s="85" t="n">
+        <x:v>2026</x:v>
+      </x:c>
+      <x:c r="E47" s="85" t="str">
+        <x:v>Amazon Web Services</x:v>
+      </x:c>
+      <x:c r="F47" s="85" t="str">
+        <x:v>AWS Savings Plans</x:v>
+      </x:c>
+      <x:c r="G47" s="85" t="str">
+        <x:v>Documentación oficial usada en FP-172 para compromisos y cobertura.</x:v>
+      </x:c>
+      <x:c r="H47" s="85" t="str">
+        <x:v>compromisos y cobertura</x:v>
+      </x:c>
+      <x:c r="I47" s="85" t="str">
+        <x:v>https://aws.amazon.com/savingsplans/</x:v>
+      </x:c>
+      <x:c r="J47" s="85" t="str">
+        <x:v>Comercial/proveedor</x:v>
+      </x:c>
+      <x:c r="K47" s="85" t="str">
+        <x:v>P2</x:v>
+      </x:c>
+      <x:c r="L47" s="85" t="str">
+        <x:v>5. Caso práctico</x:v>
+      </x:c>
+      <x:c r="M47" s="84" t="str">
+        <x:f t="shared" si="4">IF(I47="","",IF(COUNTIFS($I$6:$I$110,I47)&gt;1,IF(COUNTIFS($I$6:$I$110,I47,$K$6:$K$110,"&lt;&gt;"&amp;K47)&gt;0,"SOLAPAMIENTO: otro pilar","Duplicada en el mismo pilar"),""))</x:f>
+      </x:c>
+      <x:c r="N47" s="85" t="str">
+        <x:v>Equipo TINV-04</x:v>
+      </x:c>
+      <x:c r="O47" s="85" t="str">
+        <x:v>Verificada para matriz</x:v>
+      </x:c>
+      <x:c r="P47" s="85" t="str">
+        <x:v>Autoridad: fuente oficial. Uso: compromisos y cobertura. Límite: validar vigencia, región, SKU y contrato antes de reutilizar cifras. Consultada el 2026-09-16.</x:v>
+      </x:c>
+      <x:c r="Q47" s="85" t="str">
+        <x:v>No</x:v>
+      </x:c>
     </x:row>
     <x:row r="48" ht="15" customHeight="1">
-      <x:c r="A48" s="22" t="str">
-        <x:f t="shared" si="3"/>
-      </x:c>
-      <x:c r="B48" s="10"/>
-      <x:c r="C48" s="10"/>
-      <x:c r="D48" s="10"/>
-      <x:c r="E48" s="10"/>
-      <x:c r="F48" s="10"/>
-      <x:c r="G48" s="10"/>
-      <x:c r="H48" s="10"/>
-      <x:c r="I48" s="10"/>
-      <x:c r="J48" s="10"/>
-      <x:c r="K48" s="10"/>
-      <x:c r="L48" s="10"/>
-      <x:c r="M48" s="22" t="str">
-        <x:f t="shared" si="4"/>
-      </x:c>
-      <x:c r="N48" s="10"/>
-      <x:c r="O48" s="10"/>
-      <x:c r="P48" s="10"/>
-      <x:c r="Q48" s="10"/>
+      <x:c r="A48" s="84" t="str">
+        <x:f t="shared" si="3">IF(F48="","",TEXT(ROW()-5,"000"))</x:f>
+        <x:v>043</x:v>
+      </x:c>
+      <x:c r="B48" s="85" t="str">
+        <x:v>Sitio oficial</x:v>
+      </x:c>
+      <x:c r="C48" s="85" t="str">
+        <x:v>compromisos de uso</x:v>
+      </x:c>
+      <x:c r="D48" s="85" t="n">
+        <x:v>2026</x:v>
+      </x:c>
+      <x:c r="E48" s="85" t="str">
+        <x:v>Google Cloud</x:v>
+      </x:c>
+      <x:c r="F48" s="85" t="str">
+        <x:v>Committed use discounts</x:v>
+      </x:c>
+      <x:c r="G48" s="85" t="str">
+        <x:v>Documentación oficial usada en FP-172 para compromisos de uso.</x:v>
+      </x:c>
+      <x:c r="H48" s="85" t="str">
+        <x:v>compromisos de uso</x:v>
+      </x:c>
+      <x:c r="I48" s="85" t="str">
+        <x:v>https://cloud.google.com/docs/cuds</x:v>
+      </x:c>
+      <x:c r="J48" s="85" t="str">
+        <x:v>Comercial/proveedor</x:v>
+      </x:c>
+      <x:c r="K48" s="85" t="str">
+        <x:v>P2</x:v>
+      </x:c>
+      <x:c r="L48" s="85" t="str">
+        <x:v>5. Caso práctico</x:v>
+      </x:c>
+      <x:c r="M48" s="84" t="str">
+        <x:f t="shared" si="4">IF(I48="","",IF(COUNTIFS($I$6:$I$110,I48)&gt;1,IF(COUNTIFS($I$6:$I$110,I48,$K$6:$K$110,"&lt;&gt;"&amp;K48)&gt;0,"SOLAPAMIENTO: otro pilar","Duplicada en el mismo pilar"),""))</x:f>
+      </x:c>
+      <x:c r="N48" s="85" t="str">
+        <x:v>Equipo TINV-04</x:v>
+      </x:c>
+      <x:c r="O48" s="85" t="str">
+        <x:v>Verificada para matriz</x:v>
+      </x:c>
+      <x:c r="P48" s="85" t="str">
+        <x:v>Autoridad: fuente oficial. Uso: compromisos de uso. Límite: validar vigencia, región, SKU y contrato antes de reutilizar cifras. Consultada el 2026-09-16.</x:v>
+      </x:c>
+      <x:c r="Q48" s="85" t="str">
+        <x:v>No</x:v>
+      </x:c>
     </x:row>
     <x:row r="49" ht="15" customHeight="1">
-      <x:c r="A49" s="22" t="str">
-        <x:f t="shared" si="3"/>
-      </x:c>
-      <x:c r="B49" s="10"/>
-      <x:c r="C49" s="10"/>
-      <x:c r="D49" s="10"/>
-      <x:c r="E49" s="10"/>
-      <x:c r="F49" s="10"/>
-      <x:c r="G49" s="10"/>
-      <x:c r="H49" s="10"/>
-      <x:c r="I49" s="10"/>
-      <x:c r="J49" s="10"/>
-      <x:c r="K49" s="10"/>
-      <x:c r="L49" s="10"/>
-      <x:c r="M49" s="22" t="str">
-        <x:f t="shared" si="4"/>
-      </x:c>
-      <x:c r="N49" s="10"/>
-      <x:c r="O49" s="10"/>
-      <x:c r="P49" s="10"/>
-      <x:c r="Q49" s="10"/>
+      <x:c r="A49" s="84" t="str">
+        <x:f t="shared" si="3">IF(F49="","",TEXT(ROW()-5,"000"))</x:f>
+        <x:v>044</x:v>
+      </x:c>
+      <x:c r="B49" s="85" t="str">
+        <x:v>Sitio oficial</x:v>
+      </x:c>
+      <x:c r="C49" s="85" t="str">
+        <x:v>capacidad interrumpible</x:v>
+      </x:c>
+      <x:c r="D49" s="85" t="n">
+        <x:v>2026</x:v>
+      </x:c>
+      <x:c r="E49" s="85" t="str">
+        <x:v>Microsoft</x:v>
+      </x:c>
+      <x:c r="F49" s="85" t="str">
+        <x:v>Azure Spot Virtual Machines</x:v>
+      </x:c>
+      <x:c r="G49" s="85" t="str">
+        <x:v>Documentación oficial usada en FP-172 para capacidad interrumpible.</x:v>
+      </x:c>
+      <x:c r="H49" s="85" t="str">
+        <x:v>capacidad interrumpible</x:v>
+      </x:c>
+      <x:c r="I49" s="85" t="str">
+        <x:v>https://learn.microsoft.com/en-us/azure/virtual-machines/spot-vms</x:v>
+      </x:c>
+      <x:c r="J49" s="85" t="str">
+        <x:v>Comercial/proveedor</x:v>
+      </x:c>
+      <x:c r="K49" s="85" t="str">
+        <x:v>P2</x:v>
+      </x:c>
+      <x:c r="L49" s="85" t="str">
+        <x:v>5. Caso práctico</x:v>
+      </x:c>
+      <x:c r="M49" s="84" t="str">
+        <x:f t="shared" si="4">IF(I49="","",IF(COUNTIFS($I$6:$I$110,I49)&gt;1,IF(COUNTIFS($I$6:$I$110,I49,$K$6:$K$110,"&lt;&gt;"&amp;K49)&gt;0,"SOLAPAMIENTO: otro pilar","Duplicada en el mismo pilar"),""))</x:f>
+      </x:c>
+      <x:c r="N49" s="85" t="str">
+        <x:v>Equipo TINV-04</x:v>
+      </x:c>
+      <x:c r="O49" s="85" t="str">
+        <x:v>Verificada para matriz</x:v>
+      </x:c>
+      <x:c r="P49" s="85" t="str">
+        <x:v>Autoridad: fuente oficial. Uso: capacidad interrumpible. Límite: validar vigencia, región, SKU y contrato antes de reutilizar cifras. Consultada el 2026-09-16.</x:v>
+      </x:c>
+      <x:c r="Q49" s="85" t="str">
+        <x:v>No</x:v>
+      </x:c>
     </x:row>
     <x:row r="50" ht="15" customHeight="1">
-      <x:c r="A50" s="22" t="str">
-        <x:f t="shared" si="3"/>
-      </x:c>
-      <x:c r="B50" s="10"/>
-      <x:c r="C50" s="10"/>
-      <x:c r="D50" s="10"/>
-      <x:c r="E50" s="10"/>
-      <x:c r="F50" s="10"/>
-      <x:c r="G50" s="10"/>
-      <x:c r="H50" s="10"/>
-      <x:c r="I50" s="10"/>
-      <x:c r="J50" s="10"/>
-      <x:c r="K50" s="10"/>
-      <x:c r="L50" s="10"/>
-      <x:c r="M50" s="22" t="str">
-        <x:f t="shared" si="4"/>
-      </x:c>
-      <x:c r="N50" s="10"/>
-      <x:c r="O50" s="10"/>
-      <x:c r="P50" s="10"/>
-      <x:c r="Q50" s="10"/>
+      <x:c r="A50" s="84" t="str">
+        <x:f t="shared" si="3">IF(F50="","",TEXT(ROW()-5,"000"))</x:f>
+        <x:v>045</x:v>
+      </x:c>
+      <x:c r="B50" s="85" t="str">
+        <x:v>Sitio oficial</x:v>
+      </x:c>
+      <x:c r="C50" s="85" t="str">
+        <x:v>capacidad interrumpible</x:v>
+      </x:c>
+      <x:c r="D50" s="85" t="n">
+        <x:v>2026</x:v>
+      </x:c>
+      <x:c r="E50" s="85" t="str">
+        <x:v>Google Cloud</x:v>
+      </x:c>
+      <x:c r="F50" s="85" t="str">
+        <x:v>Spot VMs</x:v>
+      </x:c>
+      <x:c r="G50" s="85" t="str">
+        <x:v>Documentación oficial usada en FP-172 para capacidad interrumpible.</x:v>
+      </x:c>
+      <x:c r="H50" s="85" t="str">
+        <x:v>capacidad interrumpible</x:v>
+      </x:c>
+      <x:c r="I50" s="85" t="str">
+        <x:v>https://cloud.google.com/compute/docs/instances/spot</x:v>
+      </x:c>
+      <x:c r="J50" s="85" t="str">
+        <x:v>Comercial/proveedor</x:v>
+      </x:c>
+      <x:c r="K50" s="85" t="str">
+        <x:v>P2</x:v>
+      </x:c>
+      <x:c r="L50" s="85" t="str">
+        <x:v>5. Caso práctico</x:v>
+      </x:c>
+      <x:c r="M50" s="84" t="str">
+        <x:f t="shared" si="4">IF(I50="","",IF(COUNTIFS($I$6:$I$110,I50)&gt;1,IF(COUNTIFS($I$6:$I$110,I50,$K$6:$K$110,"&lt;&gt;"&amp;K50)&gt;0,"SOLAPAMIENTO: otro pilar","Duplicada en el mismo pilar"),""))</x:f>
+      </x:c>
+      <x:c r="N50" s="85" t="str">
+        <x:v>Equipo TINV-04</x:v>
+      </x:c>
+      <x:c r="O50" s="85" t="str">
+        <x:v>Verificada para matriz</x:v>
+      </x:c>
+      <x:c r="P50" s="85" t="str">
+        <x:v>Autoridad: fuente oficial. Uso: capacidad interrumpible. Límite: validar vigencia, región, SKU y contrato antes de reutilizar cifras. Consultada el 2026-09-16.</x:v>
+      </x:c>
+      <x:c r="Q50" s="85" t="str">
+        <x:v>No</x:v>
+      </x:c>
     </x:row>
     <x:row r="51" ht="15" customHeight="1">
-      <x:c r="A51" s="22" t="str">
-        <x:f t="shared" si="3"/>
-      </x:c>
-      <x:c r="B51" s="10"/>
-      <x:c r="C51" s="10"/>
-      <x:c r="D51" s="10"/>
-      <x:c r="E51" s="10"/>
-      <x:c r="F51" s="10"/>
-      <x:c r="G51" s="10"/>
-      <x:c r="H51" s="10"/>
-      <x:c r="I51" s="10"/>
-      <x:c r="J51" s="10"/>
-      <x:c r="K51" s="10"/>
-      <x:c r="L51" s="10"/>
-      <x:c r="M51" s="22" t="str">
-        <x:f t="shared" si="4"/>
-      </x:c>
-      <x:c r="N51" s="10"/>
-      <x:c r="O51" s="10"/>
-      <x:c r="P51" s="10"/>
-      <x:c r="Q51" s="10"/>
+      <x:c r="A51" s="84" t="str">
+        <x:f t="shared" si="3">IF(F51="","",TEXT(ROW()-5,"000"))</x:f>
+        <x:v>046</x:v>
+      </x:c>
+      <x:c r="B51" s="85" t="str">
+        <x:v>Sitio oficial</x:v>
+      </x:c>
+      <x:c r="C51" s="85" t="str">
+        <x:v>niveles de almacenamiento</x:v>
+      </x:c>
+      <x:c r="D51" s="85" t="n">
+        <x:v>2026</x:v>
+      </x:c>
+      <x:c r="E51" s="85" t="str">
+        <x:v>Microsoft</x:v>
+      </x:c>
+      <x:c r="F51" s="85" t="str">
+        <x:v>Access tiers for blob data</x:v>
+      </x:c>
+      <x:c r="G51" s="85" t="str">
+        <x:v>Documentación oficial usada en FP-172 para niveles de almacenamiento.</x:v>
+      </x:c>
+      <x:c r="H51" s="85" t="str">
+        <x:v>niveles de almacenamiento</x:v>
+      </x:c>
+      <x:c r="I51" s="85" t="str">
+        <x:v>https://learn.microsoft.com/en-us/azure/storage/blobs/access-tiers-overview</x:v>
+      </x:c>
+      <x:c r="J51" s="85" t="str">
+        <x:v>Comercial/proveedor</x:v>
+      </x:c>
+      <x:c r="K51" s="85" t="str">
+        <x:v>P2</x:v>
+      </x:c>
+      <x:c r="L51" s="85" t="str">
+        <x:v>5. Caso práctico</x:v>
+      </x:c>
+      <x:c r="M51" s="84" t="str">
+        <x:f t="shared" si="4">IF(I51="","",IF(COUNTIFS($I$6:$I$110,I51)&gt;1,IF(COUNTIFS($I$6:$I$110,I51,$K$6:$K$110,"&lt;&gt;"&amp;K51)&gt;0,"SOLAPAMIENTO: otro pilar","Duplicada en el mismo pilar"),""))</x:f>
+      </x:c>
+      <x:c r="N51" s="85" t="str">
+        <x:v>Equipo TINV-04</x:v>
+      </x:c>
+      <x:c r="O51" s="85" t="str">
+        <x:v>Verificada para matriz</x:v>
+      </x:c>
+      <x:c r="P51" s="85" t="str">
+        <x:v>Autoridad: fuente oficial. Uso: niveles de almacenamiento. Límite: validar vigencia, región, SKU y contrato antes de reutilizar cifras. Consultada el 2026-09-16.</x:v>
+      </x:c>
+      <x:c r="Q51" s="85" t="str">
+        <x:v>No</x:v>
+      </x:c>
     </x:row>
     <x:row r="52" ht="15" customHeight="1">
-      <x:c r="A52" s="22" t="str">
-        <x:f t="shared" si="3"/>
-      </x:c>
-      <x:c r="B52" s="10"/>
-      <x:c r="C52" s="10"/>
-      <x:c r="D52" s="10"/>
-      <x:c r="E52" s="10"/>
-      <x:c r="F52" s="10"/>
-      <x:c r="G52" s="10"/>
-      <x:c r="H52" s="10"/>
-      <x:c r="I52" s="10"/>
-      <x:c r="J52" s="10"/>
-      <x:c r="K52" s="10"/>
-      <x:c r="L52" s="10"/>
-      <x:c r="M52" s="22" t="str">
-        <x:f t="shared" si="4"/>
-      </x:c>
-      <x:c r="N52" s="10"/>
-      <x:c r="O52" s="10"/>
-      <x:c r="P52" s="10"/>
-      <x:c r="Q52" s="10"/>
+      <x:c r="A52" s="84" t="str">
+        <x:f t="shared" si="3">IF(F52="","",TEXT(ROW()-5,"000"))</x:f>
+        <x:v>047</x:v>
+      </x:c>
+      <x:c r="B52" s="85" t="str">
+        <x:v>Sitio oficial</x:v>
+      </x:c>
+      <x:c r="C52" s="85" t="str">
+        <x:v>cambios de arquitectura</x:v>
+      </x:c>
+      <x:c r="D52" s="85" t="n">
+        <x:v>2026</x:v>
+      </x:c>
+      <x:c r="E52" s="85" t="str">
+        <x:v>Microsoft</x:v>
+      </x:c>
+      <x:c r="F52" s="85" t="str">
+        <x:v>Serverless computing technology choices</x:v>
+      </x:c>
+      <x:c r="G52" s="85" t="str">
+        <x:v>Documentación oficial usada en FP-172 para cambios de arquitectura.</x:v>
+      </x:c>
+      <x:c r="H52" s="85" t="str">
+        <x:v>cambios de arquitectura</x:v>
+      </x:c>
+      <x:c r="I52" s="85" t="str">
+        <x:v>https://learn.microsoft.com/en-us/azure/architecture/guide/technology-choices/serverless-computing</x:v>
+      </x:c>
+      <x:c r="J52" s="85" t="str">
+        <x:v>Comercial/proveedor</x:v>
+      </x:c>
+      <x:c r="K52" s="85" t="str">
+        <x:v>P2</x:v>
+      </x:c>
+      <x:c r="L52" s="85" t="str">
+        <x:v>5. Caso práctico</x:v>
+      </x:c>
+      <x:c r="M52" s="84" t="str">
+        <x:f t="shared" si="4">IF(I52="","",IF(COUNTIFS($I$6:$I$110,I52)&gt;1,IF(COUNTIFS($I$6:$I$110,I52,$K$6:$K$110,"&lt;&gt;"&amp;K52)&gt;0,"SOLAPAMIENTO: otro pilar","Duplicada en el mismo pilar"),""))</x:f>
+      </x:c>
+      <x:c r="N52" s="85" t="str">
+        <x:v>Equipo TINV-04</x:v>
+      </x:c>
+      <x:c r="O52" s="85" t="str">
+        <x:v>Verificada para matriz</x:v>
+      </x:c>
+      <x:c r="P52" s="85" t="str">
+        <x:v>Autoridad: fuente oficial. Uso: cambios de arquitectura. Límite: validar vigencia, región, SKU y contrato antes de reutilizar cifras. Consultada el 2026-09-16.</x:v>
+      </x:c>
+      <x:c r="Q52" s="85" t="str">
+        <x:v>No</x:v>
+      </x:c>
     </x:row>
     <x:row r="53" ht="15" customHeight="1">
-      <x:c r="A53" s="22" t="str">
-        <x:f t="shared" si="3"/>
-      </x:c>
-      <x:c r="B53" s="10"/>
-      <x:c r="C53" s="10"/>
-      <x:c r="D53" s="10"/>
-      <x:c r="E53" s="10"/>
-      <x:c r="F53" s="10"/>
-      <x:c r="G53" s="10"/>
-      <x:c r="H53" s="10"/>
-      <x:c r="I53" s="10"/>
-      <x:c r="J53" s="10"/>
-      <x:c r="K53" s="10"/>
-      <x:c r="L53" s="10"/>
-      <x:c r="M53" s="22" t="str">
-        <x:f t="shared" si="4"/>
-      </x:c>
-      <x:c r="N53" s="10"/>
-      <x:c r="O53" s="10"/>
-      <x:c r="P53" s="10"/>
-      <x:c r="Q53" s="10"/>
+      <x:c r="A53" s="84" t="str">
+        <x:f t="shared" si="3">IF(F53="","",TEXT(ROW()-5,"000"))</x:f>
+        <x:v>048</x:v>
+      </x:c>
+      <x:c r="B53" s="85" t="str">
+        <x:v>Sitio oficial</x:v>
+      </x:c>
+      <x:c r="C53" s="85" t="str">
+        <x:v>egress e interregión</x:v>
+      </x:c>
+      <x:c r="D53" s="85" t="n">
+        <x:v>2026</x:v>
+      </x:c>
+      <x:c r="E53" s="85" t="str">
+        <x:v>Microsoft</x:v>
+      </x:c>
+      <x:c r="F53" s="85" t="str">
+        <x:v>Azure Bandwidth Pricing</x:v>
+      </x:c>
+      <x:c r="G53" s="85" t="str">
+        <x:v>Documentación oficial usada en FP-172 para egress e interregión.</x:v>
+      </x:c>
+      <x:c r="H53" s="85" t="str">
+        <x:v>egress e interregión</x:v>
+      </x:c>
+      <x:c r="I53" s="85" t="str">
+        <x:v>https://azure.microsoft.com/en-us/pricing/details/bandwidth/</x:v>
+      </x:c>
+      <x:c r="J53" s="85" t="str">
+        <x:v>Comercial/proveedor</x:v>
+      </x:c>
+      <x:c r="K53" s="85" t="str">
+        <x:v>P2</x:v>
+      </x:c>
+      <x:c r="L53" s="85" t="str">
+        <x:v>5. Caso práctico</x:v>
+      </x:c>
+      <x:c r="M53" s="84" t="str">
+        <x:f t="shared" si="4">IF(I53="","",IF(COUNTIFS($I$6:$I$110,I53)&gt;1,IF(COUNTIFS($I$6:$I$110,I53,$K$6:$K$110,"&lt;&gt;"&amp;K53)&gt;0,"SOLAPAMIENTO: otro pilar","Duplicada en el mismo pilar"),""))</x:f>
+      </x:c>
+      <x:c r="N53" s="85" t="str">
+        <x:v>Equipo TINV-04</x:v>
+      </x:c>
+      <x:c r="O53" s="85" t="str">
+        <x:v>Verificada para matriz</x:v>
+      </x:c>
+      <x:c r="P53" s="85" t="str">
+        <x:v>Autoridad: fuente oficial. Uso: egress e interregión. Límite: validar vigencia, región, SKU y contrato antes de reutilizar cifras. Consultada el 2026-09-16.</x:v>
+      </x:c>
+      <x:c r="Q53" s="85" t="str">
+        <x:v>No</x:v>
+      </x:c>
     </x:row>
     <x:row r="54" ht="15" customHeight="1">
-      <x:c r="A54" s="22" t="str">
-        <x:f t="shared" si="3"/>
-      </x:c>
-      <x:c r="B54" s="10"/>
-      <x:c r="C54" s="10"/>
-      <x:c r="D54" s="10"/>
-      <x:c r="E54" s="10"/>
-      <x:c r="F54" s="10"/>
-      <x:c r="G54" s="10"/>
-      <x:c r="H54" s="10"/>
-      <x:c r="I54" s="10"/>
-      <x:c r="J54" s="10"/>
-      <x:c r="K54" s="10"/>
-      <x:c r="L54" s="10"/>
-      <x:c r="M54" s="22" t="str">
-        <x:f t="shared" si="4"/>
-      </x:c>
-      <x:c r="N54" s="10"/>
-      <x:c r="O54" s="10"/>
-      <x:c r="P54" s="10"/>
-      <x:c r="Q54" s="10"/>
+      <x:c r="A54" s="84" t="str">
+        <x:f t="shared" si="3">IF(F54="","",TEXT(ROW()-5,"000"))</x:f>
+        <x:v>049</x:v>
+      </x:c>
+      <x:c r="B54" s="85" t="str">
+        <x:v>Sitio oficial</x:v>
+      </x:c>
+      <x:c r="C54" s="85" t="str">
+        <x:v>tráfico entre redes</x:v>
+      </x:c>
+      <x:c r="D54" s="85" t="n">
+        <x:v>2026</x:v>
+      </x:c>
+      <x:c r="E54" s="85" t="str">
+        <x:v>Microsoft</x:v>
+      </x:c>
+      <x:c r="F54" s="85" t="str">
+        <x:v>Virtual network peering</x:v>
+      </x:c>
+      <x:c r="G54" s="85" t="str">
+        <x:v>Documentación oficial usada en FP-172 para tráfico entre redes.</x:v>
+      </x:c>
+      <x:c r="H54" s="85" t="str">
+        <x:v>tráfico entre redes</x:v>
+      </x:c>
+      <x:c r="I54" s="85" t="str">
+        <x:v>https://learn.microsoft.com/en-us/azure/virtual-network/virtual-network-peering-overview</x:v>
+      </x:c>
+      <x:c r="J54" s="85" t="str">
+        <x:v>Comercial/proveedor</x:v>
+      </x:c>
+      <x:c r="K54" s="85" t="str">
+        <x:v>P2</x:v>
+      </x:c>
+      <x:c r="L54" s="85" t="str">
+        <x:v>5. Caso práctico</x:v>
+      </x:c>
+      <x:c r="M54" s="84" t="str">
+        <x:f t="shared" si="4">IF(I54="","",IF(COUNTIFS($I$6:$I$110,I54)&gt;1,IF(COUNTIFS($I$6:$I$110,I54,$K$6:$K$110,"&lt;&gt;"&amp;K54)&gt;0,"SOLAPAMIENTO: otro pilar","Duplicada en el mismo pilar"),""))</x:f>
+      </x:c>
+      <x:c r="N54" s="85" t="str">
+        <x:v>Equipo TINV-04</x:v>
+      </x:c>
+      <x:c r="O54" s="85" t="str">
+        <x:v>Verificada para matriz</x:v>
+      </x:c>
+      <x:c r="P54" s="85" t="str">
+        <x:v>Autoridad: fuente oficial. Uso: tráfico entre redes. Límite: validar vigencia, región, SKU y contrato antes de reutilizar cifras. Consultada el 2026-09-16.</x:v>
+      </x:c>
+      <x:c r="Q54" s="85" t="str">
+        <x:v>No</x:v>
+      </x:c>
     </x:row>
     <x:row r="55" ht="15" customHeight="1">
-      <x:c r="A55" s="22" t="str">
-        <x:f t="shared" si="3"/>
-      </x:c>
-      <x:c r="B55" s="10"/>
-      <x:c r="C55" s="10"/>
-      <x:c r="D55" s="10"/>
-      <x:c r="E55" s="10"/>
-      <x:c r="F55" s="10"/>
-      <x:c r="G55" s="10"/>
-      <x:c r="H55" s="10"/>
-      <x:c r="I55" s="10"/>
-      <x:c r="J55" s="10"/>
-      <x:c r="K55" s="10"/>
-      <x:c r="L55" s="10"/>
-      <x:c r="M55" s="22" t="str">
-        <x:f t="shared" si="4"/>
-      </x:c>
-      <x:c r="N55" s="10"/>
-      <x:c r="O55" s="10"/>
-      <x:c r="P55" s="10"/>
-      <x:c r="Q55" s="10"/>
+      <x:c r="A55" s="84" t="str">
+        <x:f t="shared" si="3">IF(F55="","",TEXT(ROW()-5,"000"))</x:f>
+        <x:v>050</x:v>
+      </x:c>
+      <x:c r="B55" s="85" t="str">
+        <x:v>Sitio oficial</x:v>
+      </x:c>
+      <x:c r="C55" s="85" t="str">
+        <x:v>licenciamiento</x:v>
+      </x:c>
+      <x:c r="D55" s="85" t="n">
+        <x:v>2026</x:v>
+      </x:c>
+      <x:c r="E55" s="85" t="str">
+        <x:v>Microsoft</x:v>
+      </x:c>
+      <x:c r="F55" s="85" t="str">
+        <x:v>Azure licensing models</x:v>
+      </x:c>
+      <x:c r="G55" s="85" t="str">
+        <x:v>Documentación oficial usada en FP-172 para licenciamiento.</x:v>
+      </x:c>
+      <x:c r="H55" s="85" t="str">
+        <x:v>licenciamiento</x:v>
+      </x:c>
+      <x:c r="I55" s="85" t="str">
+        <x:v>https://azure.microsoft.com/en-us/pricing/licensing-models/</x:v>
+      </x:c>
+      <x:c r="J55" s="85" t="str">
+        <x:v>Comercial/proveedor</x:v>
+      </x:c>
+      <x:c r="K55" s="85" t="str">
+        <x:v>P2</x:v>
+      </x:c>
+      <x:c r="L55" s="85" t="str">
+        <x:v>5. Caso práctico</x:v>
+      </x:c>
+      <x:c r="M55" s="84" t="str">
+        <x:f t="shared" si="4">IF(I55="","",IF(COUNTIFS($I$6:$I$110,I55)&gt;1,IF(COUNTIFS($I$6:$I$110,I55,$K$6:$K$110,"&lt;&gt;"&amp;K55)&gt;0,"SOLAPAMIENTO: otro pilar","Duplicada en el mismo pilar"),""))</x:f>
+      </x:c>
+      <x:c r="N55" s="85" t="str">
+        <x:v>Equipo TINV-04</x:v>
+      </x:c>
+      <x:c r="O55" s="85" t="str">
+        <x:v>Verificada para matriz</x:v>
+      </x:c>
+      <x:c r="P55" s="85" t="str">
+        <x:v>Autoridad: fuente oficial. Uso: licenciamiento. Límite: validar vigencia, región, SKU y contrato antes de reutilizar cifras. Consultada el 2026-09-16.</x:v>
+      </x:c>
+      <x:c r="Q55" s="85" t="str">
+        <x:v>No</x:v>
+      </x:c>
     </x:row>
     <x:row r="56" ht="15" customHeight="1">
-      <x:c r="A56" s="22" t="str">
-        <x:f t="shared" si="3"/>
-      </x:c>
-      <x:c r="B56" s="10"/>
-      <x:c r="C56" s="10"/>
-      <x:c r="D56" s="10"/>
-      <x:c r="E56" s="10"/>
-      <x:c r="F56" s="10"/>
-      <x:c r="G56" s="10"/>
-      <x:c r="H56" s="10"/>
-      <x:c r="I56" s="10"/>
-      <x:c r="J56" s="10"/>
-      <x:c r="K56" s="10"/>
-      <x:c r="L56" s="10"/>
-      <x:c r="M56" s="22" t="str">
-        <x:f t="shared" si="4"/>
-      </x:c>
-      <x:c r="N56" s="10"/>
-      <x:c r="O56" s="10"/>
-      <x:c r="P56" s="10"/>
-      <x:c r="Q56" s="10"/>
+      <x:c r="A56" s="84" t="str">
+        <x:f t="shared" si="3">IF(F56="","",TEXT(ROW()-5,"000"))</x:f>
+        <x:v>051</x:v>
+      </x:c>
+      <x:c r="B56" s="85" t="str">
+        <x:v>Sitio oficial</x:v>
+      </x:c>
+      <x:c r="C56" s="85" t="str">
+        <x:v>niveles de soporte</x:v>
+      </x:c>
+      <x:c r="D56" s="85" t="n">
+        <x:v>2026</x:v>
+      </x:c>
+      <x:c r="E56" s="85" t="str">
+        <x:v>Microsoft</x:v>
+      </x:c>
+      <x:c r="F56" s="85" t="str">
+        <x:v>Azure support plans</x:v>
+      </x:c>
+      <x:c r="G56" s="85" t="str">
+        <x:v>Documentación oficial usada en FP-172 para niveles de soporte.</x:v>
+      </x:c>
+      <x:c r="H56" s="85" t="str">
+        <x:v>niveles de soporte</x:v>
+      </x:c>
+      <x:c r="I56" s="85" t="str">
+        <x:v>https://azure.microsoft.com/en-us/support/plans/</x:v>
+      </x:c>
+      <x:c r="J56" s="85" t="str">
+        <x:v>Comercial/proveedor</x:v>
+      </x:c>
+      <x:c r="K56" s="85" t="str">
+        <x:v>P2</x:v>
+      </x:c>
+      <x:c r="L56" s="85" t="str">
+        <x:v>5. Caso práctico</x:v>
+      </x:c>
+      <x:c r="M56" s="84" t="str">
+        <x:f t="shared" si="4">IF(I56="","",IF(COUNTIFS($I$6:$I$110,I56)&gt;1,IF(COUNTIFS($I$6:$I$110,I56,$K$6:$K$110,"&lt;&gt;"&amp;K56)&gt;0,"SOLAPAMIENTO: otro pilar","Duplicada en el mismo pilar"),""))</x:f>
+      </x:c>
+      <x:c r="N56" s="85" t="str">
+        <x:v>Equipo TINV-04</x:v>
+      </x:c>
+      <x:c r="O56" s="85" t="str">
+        <x:v>Verificada para matriz</x:v>
+      </x:c>
+      <x:c r="P56" s="85" t="str">
+        <x:v>Autoridad: fuente oficial. Uso: niveles de soporte. Límite: validar vigencia, región, SKU y contrato antes de reutilizar cifras. Consultada el 2026-09-16.</x:v>
+      </x:c>
+      <x:c r="Q56" s="85" t="str">
+        <x:v>No</x:v>
+      </x:c>
     </x:row>
     <x:row r="57" ht="15" customHeight="1">
-      <x:c r="A57" s="22" t="str">
-        <x:f t="shared" si="3"/>
-      </x:c>
-      <x:c r="B57" s="10"/>
-      <x:c r="C57" s="10"/>
-      <x:c r="D57" s="10"/>
-      <x:c r="E57" s="10"/>
-      <x:c r="F57" s="10"/>
-      <x:c r="G57" s="10"/>
-      <x:c r="H57" s="10"/>
-      <x:c r="I57" s="10"/>
-      <x:c r="J57" s="10"/>
-      <x:c r="K57" s="10"/>
-      <x:c r="L57" s="10"/>
-      <x:c r="M57" s="22" t="str">
-        <x:f t="shared" si="4"/>
-      </x:c>
-      <x:c r="N57" s="10"/>
-      <x:c r="O57" s="10"/>
-      <x:c r="P57" s="10"/>
-      <x:c r="Q57" s="10"/>
+      <x:c r="A57" s="84" t="str">
+        <x:f t="shared" si="3">IF(F57="","",TEXT(ROW()-5,"000"))</x:f>
+        <x:v>052</x:v>
+      </x:c>
+      <x:c r="B57" s="85" t="str">
+        <x:v>Sitio oficial</x:v>
+      </x:c>
+      <x:c r="C57" s="85" t="str">
+        <x:v>ambientes no productivos</x:v>
+      </x:c>
+      <x:c r="D57" s="85" t="n">
+        <x:v>2026</x:v>
+      </x:c>
+      <x:c r="E57" s="85" t="str">
+        <x:v>Microsoft</x:v>
+      </x:c>
+      <x:c r="F57" s="85" t="str">
+        <x:v>Auto-shutdown for Azure VMs</x:v>
+      </x:c>
+      <x:c r="G57" s="85" t="str">
+        <x:v>Documentación oficial usada en FP-172 para ambientes no productivos.</x:v>
+      </x:c>
+      <x:c r="H57" s="85" t="str">
+        <x:v>ambientes no productivos</x:v>
+      </x:c>
+      <x:c r="I57" s="85" t="str">
+        <x:v>https://learn.microsoft.com/en-us/azure/virtual-machines/auto-shutdown-vm</x:v>
+      </x:c>
+      <x:c r="J57" s="85" t="str">
+        <x:v>Comercial/proveedor</x:v>
+      </x:c>
+      <x:c r="K57" s="85" t="str">
+        <x:v>P2</x:v>
+      </x:c>
+      <x:c r="L57" s="85" t="str">
+        <x:v>5. Caso práctico</x:v>
+      </x:c>
+      <x:c r="M57" s="84" t="str">
+        <x:f t="shared" si="4">IF(I57="","",IF(COUNTIFS($I$6:$I$110,I57)&gt;1,IF(COUNTIFS($I$6:$I$110,I57,$K$6:$K$110,"&lt;&gt;"&amp;K57)&gt;0,"SOLAPAMIENTO: otro pilar","Duplicada en el mismo pilar"),""))</x:f>
+      </x:c>
+      <x:c r="N57" s="85" t="str">
+        <x:v>Equipo TINV-04</x:v>
+      </x:c>
+      <x:c r="O57" s="85" t="str">
+        <x:v>Verificada para matriz</x:v>
+      </x:c>
+      <x:c r="P57" s="85" t="str">
+        <x:v>Autoridad: fuente oficial. Uso: ambientes no productivos. Límite: validar vigencia, región, SKU y contrato antes de reutilizar cifras. Consultada el 2026-09-16.</x:v>
+      </x:c>
+      <x:c r="Q57" s="85" t="str">
+        <x:v>No</x:v>
+      </x:c>
     </x:row>
     <x:row r="58" ht="15" customHeight="1">
-      <x:c r="A58" s="22" t="str">
-        <x:f t="shared" si="3"/>
-      </x:c>
-      <x:c r="B58" s="10"/>
-      <x:c r="C58" s="10"/>
-      <x:c r="D58" s="10"/>
-      <x:c r="E58" s="10"/>
-      <x:c r="F58" s="10"/>
-      <x:c r="G58" s="10"/>
-      <x:c r="H58" s="10"/>
-      <x:c r="I58" s="10"/>
-      <x:c r="J58" s="10"/>
-      <x:c r="K58" s="10"/>
-      <x:c r="L58" s="10"/>
-      <x:c r="M58" s="22" t="str">
-        <x:f t="shared" si="4"/>
-      </x:c>
-      <x:c r="N58" s="10"/>
-      <x:c r="O58" s="10"/>
-      <x:c r="P58" s="10"/>
-      <x:c r="Q58" s="10"/>
+      <x:c r="A58" s="84" t="str">
+        <x:f t="shared" si="3">IF(F58="","",TEXT(ROW()-5,"000"))</x:f>
+        <x:v>053</x:v>
+      </x:c>
+      <x:c r="B58" s="85" t="str">
+        <x:v>Sitio oficial</x:v>
+      </x:c>
+      <x:c r="C58" s="85" t="str">
+        <x:v>backup automático y tarifa</x:v>
+      </x:c>
+      <x:c r="D58" s="85" t="n">
+        <x:v>2026</x:v>
+      </x:c>
+      <x:c r="E58" s="85" t="str">
+        <x:v>Microsoft</x:v>
+      </x:c>
+      <x:c r="F58" s="85" t="str">
+        <x:v>Azure Database for PostgreSQL pricing</x:v>
+      </x:c>
+      <x:c r="G58" s="85" t="str">
+        <x:v>Documentación oficial usada en FP-172 para backup automático y tarifa.</x:v>
+      </x:c>
+      <x:c r="H58" s="85" t="str">
+        <x:v>backup automático y tarifa</x:v>
+      </x:c>
+      <x:c r="I58" s="85" t="str">
+        <x:v>https://azure.microsoft.com/en-us/pricing/details/postgresql/flexible-server/</x:v>
+      </x:c>
+      <x:c r="J58" s="85" t="str">
+        <x:v>Comercial/proveedor</x:v>
+      </x:c>
+      <x:c r="K58" s="85" t="str">
+        <x:v>P2</x:v>
+      </x:c>
+      <x:c r="L58" s="85" t="str">
+        <x:v>5. Caso práctico</x:v>
+      </x:c>
+      <x:c r="M58" s="84" t="str">
+        <x:f t="shared" si="4">IF(I58="","",IF(COUNTIFS($I$6:$I$110,I58)&gt;1,IF(COUNTIFS($I$6:$I$110,I58,$K$6:$K$110,"&lt;&gt;"&amp;K58)&gt;0,"SOLAPAMIENTO: otro pilar","Duplicada en el mismo pilar"),""))</x:f>
+      </x:c>
+      <x:c r="N58" s="85" t="str">
+        <x:v>Equipo TINV-04</x:v>
+      </x:c>
+      <x:c r="O58" s="85" t="str">
+        <x:v>Verificada para matriz</x:v>
+      </x:c>
+      <x:c r="P58" s="85" t="str">
+        <x:v>Autoridad: fuente oficial. Uso: backup automático y tarifa. Límite: validar vigencia, región, SKU y contrato antes de reutilizar cifras. Consultada el 2026-09-16.</x:v>
+      </x:c>
+      <x:c r="Q58" s="85" t="str">
+        <x:v>No</x:v>
+      </x:c>
     </x:row>
     <x:row r="59" ht="15" customHeight="1">
-      <x:c r="A59" s="22" t="str">
-        <x:f t="shared" si="3"/>
-      </x:c>
-      <x:c r="B59" s="10"/>
-      <x:c r="C59" s="10"/>
-      <x:c r="D59" s="10"/>
-      <x:c r="E59" s="10"/>
-      <x:c r="F59" s="10"/>
-      <x:c r="G59" s="10"/>
-      <x:c r="H59" s="10"/>
-      <x:c r="I59" s="10"/>
-      <x:c r="J59" s="10"/>
-      <x:c r="K59" s="10"/>
-      <x:c r="L59" s="10"/>
-      <x:c r="M59" s="22" t="str">
-        <x:f t="shared" si="4"/>
-      </x:c>
-      <x:c r="N59" s="10"/>
-      <x:c r="O59" s="10"/>
-      <x:c r="P59" s="10"/>
-      <x:c r="Q59" s="10"/>
+      <x:c r="A59" s="84" t="str">
+        <x:f t="shared" si="3">IF(F59="","",TEXT(ROW()-5,"000"))</x:f>
+        <x:v>054</x:v>
+      </x:c>
+      <x:c r="B59" s="85" t="str">
+        <x:v>Sitio oficial</x:v>
+      </x:c>
+      <x:c r="C59" s="85" t="str">
+        <x:v>ingesta, retención y consultas</x:v>
+      </x:c>
+      <x:c r="D59" s="85" t="n">
+        <x:v>2026</x:v>
+      </x:c>
+      <x:c r="E59" s="85" t="str">
+        <x:v>Microsoft</x:v>
+      </x:c>
+      <x:c r="F59" s="85" t="str">
+        <x:v>Azure Monitor Logs cost</x:v>
+      </x:c>
+      <x:c r="G59" s="85" t="str">
+        <x:v>Documentación oficial usada en FP-172 para ingesta, retención y consultas.</x:v>
+      </x:c>
+      <x:c r="H59" s="85" t="str">
+        <x:v>ingesta, retención y consultas</x:v>
+      </x:c>
+      <x:c r="I59" s="85" t="str">
+        <x:v>https://learn.microsoft.com/en-us/azure/azure-monitor/logs/cost-logs</x:v>
+      </x:c>
+      <x:c r="J59" s="85" t="str">
+        <x:v>Comercial/proveedor</x:v>
+      </x:c>
+      <x:c r="K59" s="85" t="str">
+        <x:v>P2</x:v>
+      </x:c>
+      <x:c r="L59" s="85" t="str">
+        <x:v>5. Caso práctico</x:v>
+      </x:c>
+      <x:c r="M59" s="84" t="str">
+        <x:f t="shared" si="4">IF(I59="","",IF(COUNTIFS($I$6:$I$110,I59)&gt;1,IF(COUNTIFS($I$6:$I$110,I59,$K$6:$K$110,"&lt;&gt;"&amp;K59)&gt;0,"SOLAPAMIENTO: otro pilar","Duplicada en el mismo pilar"),""))</x:f>
+      </x:c>
+      <x:c r="N59" s="85" t="str">
+        <x:v>Equipo TINV-04</x:v>
+      </x:c>
+      <x:c r="O59" s="85" t="str">
+        <x:v>Verificada para matriz</x:v>
+      </x:c>
+      <x:c r="P59" s="85" t="str">
+        <x:v>Autoridad: fuente oficial. Uso: ingesta, retención y consultas. Límite: validar vigencia, región, SKU y contrato antes de reutilizar cifras. Consultada el 2026-09-16.</x:v>
+      </x:c>
+      <x:c r="Q59" s="85" t="str">
+        <x:v>No</x:v>
+      </x:c>
     </x:row>
     <x:row r="60" ht="15" customHeight="1">
       <x:c r="A60" s="22" t="str">
@@ -13377,7 +13845,7 @@
       </x:c>
       <x:c r="C7" s="23" t="n">
         <x:f>COUNTIFS('Matriz de Fuentes'!$K$6:$K$110,$A7,'Matriz de Fuentes'!$J$6:$J$110,"&lt;&gt;Academica",'Matriz de Fuentes'!$J$6:$J$110,"&lt;&gt;")</x:f>
-        <x:v>11</x:v>
+        <x:v>26</x:v>
       </x:c>
       <x:c r="D7" s="23">
         <x:f t="shared" si="1"/>
@@ -13500,7 +13968,7 @@
       </x:c>
       <x:c r="B14" s="21" t="n">
         <x:f>COUNTIFS('Matriz de Fuentes'!$J$6:$J$110,"&lt;&gt;Academica",'Matriz de Fuentes'!$J$6:$J$110,"&lt;&gt;")</x:f>
-        <x:v>26</x:v>
+        <x:v>41</x:v>
       </x:c>
       <x:c r="C14" s="35" t="s">
         <x:v>367</x:v>
@@ -13784,11 +14252,11 @@
       <x:c r="A34" s="41" t="s">
         <x:v>386</x:v>
       </x:c>
-      <x:c r="B34" s="42" t="s">
+      <x:c r="B34" s="42" t="str">
+        <x:v>Actualización 2026-09-15: se incorporaron 12 precios Azure (seis categorías por región) desde Azure Retail Prices API. Mantener validación humana de SKU y contrato.</x:v>
+      </x:c>
+      <x:c r="C34" s="43" t="s">
         <x:v>387</x:v>
-      </x:c>
-      <x:c r="C34" s="43" t="s">
-        <x:v>388</x:v>
       </x:c>
       <x:c r="D34" s="44"/>
       <x:c r="E34" s="44"/>
@@ -13796,13 +14264,13 @@
     </x:row>
     <x:row r="35" ht="54" customHeight="1">
       <x:c r="A35" s="41" t="s">
+        <x:v>388</x:v>
+      </x:c>
+      <x:c r="B35" s="42" t="s">
         <x:v>389</x:v>
       </x:c>
-      <x:c r="B35" s="42" t="s">
+      <x:c r="C35" s="43" t="s">
         <x:v>390</x:v>
-      </x:c>
-      <x:c r="C35" s="43" t="s">
-        <x:v>391</x:v>
       </x:c>
       <x:c r="D35" s="44"/>
       <x:c r="E35" s="44"/>
@@ -16198,12 +16666,12 @@
   <x:sheetData>
     <x:row r="1" ht="17.25" customHeight="1">
       <x:c r="A1" s="1" t="s">
-        <x:v>392</x:v>
+        <x:v>391</x:v>
       </x:c>
     </x:row>
     <x:row r="2" ht="15" customHeight="1">
       <x:c r="A2" s="2" t="s">
-        <x:v>393</x:v>
+        <x:v>392</x:v>
       </x:c>
     </x:row>
     <x:row r="3">
@@ -16218,7 +16686,7 @@
     </x:row>
     <x:row r="4" ht="27.75" customHeight="1">
       <x:c r="A4" s="5" t="s">
-        <x:v>394</x:v>
+        <x:v>393</x:v>
       </x:c>
       <x:c r="B4" s="5" t="s">
         <x:v>353</x:v>
@@ -16227,22 +16695,22 @@
         <x:v>65</x:v>
       </x:c>
       <x:c r="D4" s="5" t="s">
+        <x:v>394</x:v>
+      </x:c>
+      <x:c r="E4" s="5" t="s">
         <x:v>395</x:v>
       </x:c>
-      <x:c r="E4" s="5" t="s">
+      <x:c r="F4" s="5" t="s">
         <x:v>396</x:v>
       </x:c>
-      <x:c r="F4" s="5" t="s">
+      <x:c r="G4" s="5" t="s">
         <x:v>397</x:v>
       </x:c>
-      <x:c r="G4" s="5" t="s">
+      <x:c r="H4" s="5" t="s">
         <x:v>398</x:v>
       </x:c>
-      <x:c r="H4" s="5" t="s">
+      <x:c r="I4" s="5" t="s">
         <x:v>399</x:v>
-      </x:c>
-      <x:c r="I4" s="5" t="s">
-        <x:v>400</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="43.5" customHeight="1">
@@ -16254,10 +16722,10 @@
         <x:v>359</x:v>
       </x:c>
       <x:c r="C5" s="13" t="s">
+        <x:v>400</x:v>
+      </x:c>
+      <x:c r="D5" s="15" t="s">
         <x:v>401</x:v>
-      </x:c>
-      <x:c r="D5" s="15" t="s">
-        <x:v>402</x:v>
       </x:c>
       <x:c r="E5" s="16">
         <x:v>46268.0</x:v>
@@ -16281,10 +16749,10 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="C6" s="13" t="s">
+        <x:v>402</x:v>
+      </x:c>
+      <x:c r="D6" s="15" t="s">
         <x:v>403</x:v>
-      </x:c>
-      <x:c r="D6" s="15" t="s">
-        <x:v>404</x:v>
       </x:c>
       <x:c r="E6" s="13"/>
       <x:c r="F6" s="13"/>
@@ -16303,7 +16771,7 @@
         <x:v>82</x:v>
       </x:c>
       <x:c r="D7" s="15" t="s">
-        <x:v>405</x:v>
+        <x:v>404</x:v>
       </x:c>
       <x:c r="E7" s="13"/>
       <x:c r="F7" s="13"/>
@@ -16319,10 +16787,10 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="C8" s="13" t="s">
+        <x:v>405</x:v>
+      </x:c>
+      <x:c r="D8" s="15" t="s">
         <x:v>406</x:v>
-      </x:c>
-      <x:c r="D8" s="15" t="s">
-        <x:v>407</x:v>
       </x:c>
       <x:c r="E8" s="13"/>
       <x:c r="F8" s="13"/>
@@ -16338,10 +16806,10 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="C9" s="13" t="s">
-        <x:v>401</x:v>
+        <x:v>400</x:v>
       </x:c>
       <x:c r="D9" s="15" t="s">
-        <x:v>407</x:v>
+        <x:v>406</x:v>
       </x:c>
       <x:c r="E9" s="13"/>
       <x:c r="F9" s="13"/>
@@ -16357,10 +16825,10 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="C10" s="13" t="s">
+        <x:v>407</x:v>
+      </x:c>
+      <x:c r="D10" s="15" t="s">
         <x:v>408</x:v>
-      </x:c>
-      <x:c r="D10" s="15" t="s">
-        <x:v>409</x:v>
       </x:c>
       <x:c r="E10" s="13"/>
       <x:c r="F10" s="13"/>
@@ -16376,10 +16844,10 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="C11" s="13" t="s">
-        <x:v>403</x:v>
+        <x:v>402</x:v>
       </x:c>
       <x:c r="D11" s="15" t="s">
-        <x:v>410</x:v>
+        <x:v>409</x:v>
       </x:c>
       <x:c r="E11" s="13"/>
       <x:c r="F11" s="13"/>
@@ -16398,7 +16866,7 @@
         <x:v>82</x:v>
       </x:c>
       <x:c r="D12" s="15" t="s">
-        <x:v>411</x:v>
+        <x:v>410</x:v>
       </x:c>
       <x:c r="E12" s="13"/>
       <x:c r="F12" s="13"/>
@@ -16414,10 +16882,10 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="C13" s="13" t="s">
-        <x:v>406</x:v>
+        <x:v>405</x:v>
       </x:c>
       <x:c r="D13" s="15" t="s">
-        <x:v>412</x:v>
+        <x:v>411</x:v>
       </x:c>
       <x:c r="E13" s="13"/>
       <x:c r="F13" s="13"/>
@@ -16433,10 +16901,10 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="C14" s="13" t="s">
-        <x:v>401</x:v>
+        <x:v>400</x:v>
       </x:c>
       <x:c r="D14" s="15" t="s">
-        <x:v>412</x:v>
+        <x:v>411</x:v>
       </x:c>
       <x:c r="E14" s="13"/>
       <x:c r="F14" s="13"/>
@@ -16452,10 +16920,10 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="C15" s="13" t="s">
-        <x:v>408</x:v>
+        <x:v>407</x:v>
       </x:c>
       <x:c r="D15" s="15" t="s">
-        <x:v>413</x:v>
+        <x:v>412</x:v>
       </x:c>
       <x:c r="E15" s="13"/>
       <x:c r="F15" s="13"/>
@@ -16471,10 +16939,10 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="C16" s="13" t="s">
-        <x:v>403</x:v>
+        <x:v>402</x:v>
       </x:c>
       <x:c r="D16" s="15" t="s">
-        <x:v>414</x:v>
+        <x:v>413</x:v>
       </x:c>
       <x:c r="E16" s="13"/>
       <x:c r="F16" s="13"/>
@@ -16493,7 +16961,7 @@
         <x:v>82</x:v>
       </x:c>
       <x:c r="D17" s="15" t="s">
-        <x:v>415</x:v>
+        <x:v>414</x:v>
       </x:c>
       <x:c r="E17" s="13"/>
       <x:c r="F17" s="13"/>
@@ -16509,10 +16977,10 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="C18" s="13" t="s">
-        <x:v>406</x:v>
+        <x:v>405</x:v>
       </x:c>
       <x:c r="D18" s="15" t="s">
-        <x:v>416</x:v>
+        <x:v>415</x:v>
       </x:c>
       <x:c r="E18" s="13"/>
       <x:c r="F18" s="13"/>
@@ -16528,10 +16996,10 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="C19" s="13" t="s">
-        <x:v>401</x:v>
+        <x:v>400</x:v>
       </x:c>
       <x:c r="D19" s="15" t="s">
-        <x:v>416</x:v>
+        <x:v>415</x:v>
       </x:c>
       <x:c r="E19" s="13"/>
       <x:c r="F19" s="13"/>
@@ -16547,10 +17015,10 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="C20" s="13" t="s">
-        <x:v>408</x:v>
+        <x:v>407</x:v>
       </x:c>
       <x:c r="D20" s="15" t="s">
-        <x:v>417</x:v>
+        <x:v>416</x:v>
       </x:c>
       <x:c r="E20" s="13"/>
       <x:c r="F20" s="13"/>
@@ -16566,10 +17034,10 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="C21" s="13" t="s">
-        <x:v>403</x:v>
+        <x:v>402</x:v>
       </x:c>
       <x:c r="D21" s="15" t="s">
-        <x:v>418</x:v>
+        <x:v>417</x:v>
       </x:c>
       <x:c r="E21" s="13"/>
       <x:c r="F21" s="13"/>
@@ -16588,7 +17056,7 @@
         <x:v>82</x:v>
       </x:c>
       <x:c r="D22" s="15" t="s">
-        <x:v>419</x:v>
+        <x:v>418</x:v>
       </x:c>
       <x:c r="E22" s="13"/>
       <x:c r="F22" s="13"/>
@@ -16604,10 +17072,10 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="C23" s="13" t="s">
-        <x:v>406</x:v>
+        <x:v>405</x:v>
       </x:c>
       <x:c r="D23" s="15" t="s">
-        <x:v>420</x:v>
+        <x:v>419</x:v>
       </x:c>
       <x:c r="E23" s="13"/>
       <x:c r="F23" s="13"/>
@@ -16623,10 +17091,10 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="C24" s="13" t="s">
-        <x:v>401</x:v>
+        <x:v>400</x:v>
       </x:c>
       <x:c r="D24" s="15" t="s">
-        <x:v>420</x:v>
+        <x:v>419</x:v>
       </x:c>
       <x:c r="E24" s="13"/>
       <x:c r="F24" s="13"/>
@@ -16642,10 +17110,10 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="C25" s="13" t="s">
-        <x:v>408</x:v>
+        <x:v>407</x:v>
       </x:c>
       <x:c r="D25" s="15" t="s">
-        <x:v>421</x:v>
+        <x:v>420</x:v>
       </x:c>
       <x:c r="E25" s="13"/>
       <x:c r="F25" s="13"/>
@@ -16661,10 +17129,10 @@
         <x:v>9</x:v>
       </x:c>
       <x:c r="C26" s="13" t="s">
-        <x:v>403</x:v>
+        <x:v>402</x:v>
       </x:c>
       <x:c r="D26" s="15" t="s">
-        <x:v>422</x:v>
+        <x:v>421</x:v>
       </x:c>
       <x:c r="E26" s="13"/>
       <x:c r="F26" s="13"/>
@@ -16683,7 +17151,7 @@
         <x:v>82</x:v>
       </x:c>
       <x:c r="D27" s="15" t="s">
-        <x:v>423</x:v>
+        <x:v>422</x:v>
       </x:c>
       <x:c r="E27" s="13"/>
       <x:c r="F27" s="13"/>
@@ -16699,10 +17167,10 @@
         <x:v>9</x:v>
       </x:c>
       <x:c r="C28" s="13" t="s">
-        <x:v>406</x:v>
+        <x:v>405</x:v>
       </x:c>
       <x:c r="D28" s="15" t="s">
-        <x:v>424</x:v>
+        <x:v>423</x:v>
       </x:c>
       <x:c r="E28" s="13"/>
       <x:c r="F28" s="13"/>
@@ -16718,10 +17186,10 @@
         <x:v>9</x:v>
       </x:c>
       <x:c r="C29" s="13" t="s">
-        <x:v>401</x:v>
+        <x:v>400</x:v>
       </x:c>
       <x:c r="D29" s="15" t="s">
-        <x:v>424</x:v>
+        <x:v>423</x:v>
       </x:c>
       <x:c r="E29" s="13"/>
       <x:c r="F29" s="13"/>
@@ -16737,10 +17205,10 @@
         <x:v>9</x:v>
       </x:c>
       <x:c r="C30" s="13" t="s">
-        <x:v>408</x:v>
+        <x:v>407</x:v>
       </x:c>
       <x:c r="D30" s="15" t="s">
-        <x:v>425</x:v>
+        <x:v>424</x:v>
       </x:c>
       <x:c r="E30" s="13"/>
       <x:c r="F30" s="13"/>
@@ -16756,10 +17224,10 @@
         <x:v>9</x:v>
       </x:c>
       <x:c r="C31" s="13" t="s">
-        <x:v>403</x:v>
+        <x:v>402</x:v>
       </x:c>
       <x:c r="D31" s="15" t="s">
-        <x:v>426</x:v>
+        <x:v>425</x:v>
       </x:c>
       <x:c r="E31" s="13"/>
       <x:c r="F31" s="13"/>
@@ -16778,7 +17246,7 @@
         <x:v>82</x:v>
       </x:c>
       <x:c r="D32" s="15" t="s">
-        <x:v>427</x:v>
+        <x:v>426</x:v>
       </x:c>
       <x:c r="E32" s="13"/>
       <x:c r="F32" s="13"/>
@@ -16794,10 +17262,10 @@
         <x:v>9</x:v>
       </x:c>
       <x:c r="C33" s="13" t="s">
-        <x:v>406</x:v>
+        <x:v>405</x:v>
       </x:c>
       <x:c r="D33" s="15" t="s">
-        <x:v>428</x:v>
+        <x:v>427</x:v>
       </x:c>
       <x:c r="E33" s="13"/>
       <x:c r="F33" s="13"/>
@@ -16813,10 +17281,10 @@
         <x:v>9</x:v>
       </x:c>
       <x:c r="C34" s="13" t="s">
-        <x:v>401</x:v>
+        <x:v>400</x:v>
       </x:c>
       <x:c r="D34" s="15" t="s">
-        <x:v>428</x:v>
+        <x:v>427</x:v>
       </x:c>
       <x:c r="E34" s="13"/>
       <x:c r="F34" s="13"/>
@@ -16832,10 +17300,10 @@
         <x:v>9</x:v>
       </x:c>
       <x:c r="C35" s="13" t="s">
-        <x:v>408</x:v>
+        <x:v>407</x:v>
       </x:c>
       <x:c r="D35" s="15" t="s">
-        <x:v>429</x:v>
+        <x:v>428</x:v>
       </x:c>
       <x:c r="E35" s="13"/>
       <x:c r="F35" s="13"/>
@@ -16851,10 +17319,10 @@
         <x:v>9</x:v>
       </x:c>
       <x:c r="C36" s="13" t="s">
-        <x:v>403</x:v>
+        <x:v>402</x:v>
       </x:c>
       <x:c r="D36" s="15" t="s">
-        <x:v>430</x:v>
+        <x:v>429</x:v>
       </x:c>
       <x:c r="E36" s="13"/>
       <x:c r="F36" s="13"/>
@@ -16873,7 +17341,7 @@
         <x:v>82</x:v>
       </x:c>
       <x:c r="D37" s="15" t="s">
-        <x:v>431</x:v>
+        <x:v>430</x:v>
       </x:c>
       <x:c r="E37" s="13"/>
       <x:c r="F37" s="13"/>
@@ -16889,10 +17357,10 @@
         <x:v>9</x:v>
       </x:c>
       <x:c r="C38" s="13" t="s">
-        <x:v>406</x:v>
+        <x:v>405</x:v>
       </x:c>
       <x:c r="D38" s="15" t="s">
-        <x:v>432</x:v>
+        <x:v>431</x:v>
       </x:c>
       <x:c r="E38" s="13"/>
       <x:c r="F38" s="13"/>
@@ -16908,10 +17376,10 @@
         <x:v>9</x:v>
       </x:c>
       <x:c r="C39" s="13" t="s">
-        <x:v>401</x:v>
+        <x:v>400</x:v>
       </x:c>
       <x:c r="D39" s="15" t="s">
-        <x:v>432</x:v>
+        <x:v>431</x:v>
       </x:c>
       <x:c r="E39" s="13"/>
       <x:c r="F39" s="13"/>
@@ -16927,10 +17395,10 @@
         <x:v>9</x:v>
       </x:c>
       <x:c r="C40" s="13" t="s">
-        <x:v>408</x:v>
+        <x:v>407</x:v>
       </x:c>
       <x:c r="D40" s="15" t="s">
-        <x:v>433</x:v>
+        <x:v>432</x:v>
       </x:c>
       <x:c r="E40" s="13"/>
       <x:c r="F40" s="13"/>
@@ -16946,10 +17414,10 @@
         <x:v>13</x:v>
       </x:c>
       <x:c r="C41" s="13" t="s">
-        <x:v>403</x:v>
+        <x:v>402</x:v>
       </x:c>
       <x:c r="D41" s="15" t="s">
-        <x:v>434</x:v>
+        <x:v>433</x:v>
       </x:c>
       <x:c r="E41" s="13"/>
       <x:c r="F41" s="13"/>
@@ -16968,7 +17436,7 @@
         <x:v>82</x:v>
       </x:c>
       <x:c r="D42" s="15" t="s">
-        <x:v>435</x:v>
+        <x:v>434</x:v>
       </x:c>
       <x:c r="E42" s="13"/>
       <x:c r="F42" s="13"/>
@@ -16984,10 +17452,10 @@
         <x:v>13</x:v>
       </x:c>
       <x:c r="C43" s="13" t="s">
-        <x:v>406</x:v>
+        <x:v>405</x:v>
       </x:c>
       <x:c r="D43" s="15" t="s">
-        <x:v>436</x:v>
+        <x:v>435</x:v>
       </x:c>
       <x:c r="E43" s="13"/>
       <x:c r="F43" s="13"/>
@@ -17003,10 +17471,10 @@
         <x:v>13</x:v>
       </x:c>
       <x:c r="C44" s="13" t="s">
-        <x:v>401</x:v>
+        <x:v>400</x:v>
       </x:c>
       <x:c r="D44" s="15" t="s">
-        <x:v>436</x:v>
+        <x:v>435</x:v>
       </x:c>
       <x:c r="E44" s="13"/>
       <x:c r="F44" s="13"/>
@@ -17022,10 +17490,10 @@
         <x:v>13</x:v>
       </x:c>
       <x:c r="C45" s="13" t="s">
-        <x:v>408</x:v>
+        <x:v>407</x:v>
       </x:c>
       <x:c r="D45" s="15" t="s">
-        <x:v>437</x:v>
+        <x:v>436</x:v>
       </x:c>
       <x:c r="E45" s="13"/>
       <x:c r="F45" s="13"/>
@@ -17041,10 +17509,10 @@
         <x:v>13</x:v>
       </x:c>
       <x:c r="C46" s="13" t="s">
-        <x:v>403</x:v>
+        <x:v>402</x:v>
       </x:c>
       <x:c r="D46" s="15" t="s">
-        <x:v>438</x:v>
+        <x:v>437</x:v>
       </x:c>
       <x:c r="E46" s="13"/>
       <x:c r="F46" s="13"/>
@@ -17063,7 +17531,7 @@
         <x:v>82</x:v>
       </x:c>
       <x:c r="D47" s="15" t="s">
-        <x:v>439</x:v>
+        <x:v>438</x:v>
       </x:c>
       <x:c r="E47" s="13"/>
       <x:c r="F47" s="13"/>
@@ -17079,10 +17547,10 @@
         <x:v>13</x:v>
       </x:c>
       <x:c r="C48" s="13" t="s">
-        <x:v>406</x:v>
+        <x:v>405</x:v>
       </x:c>
       <x:c r="D48" s="15" t="s">
-        <x:v>440</x:v>
+        <x:v>439</x:v>
       </x:c>
       <x:c r="E48" s="13"/>
       <x:c r="F48" s="13"/>
@@ -17098,10 +17566,10 @@
         <x:v>13</x:v>
       </x:c>
       <x:c r="C49" s="13" t="s">
-        <x:v>401</x:v>
+        <x:v>400</x:v>
       </x:c>
       <x:c r="D49" s="15" t="s">
-        <x:v>440</x:v>
+        <x:v>439</x:v>
       </x:c>
       <x:c r="E49" s="13"/>
       <x:c r="F49" s="13"/>
@@ -17117,10 +17585,10 @@
         <x:v>13</x:v>
       </x:c>
       <x:c r="C50" s="13" t="s">
-        <x:v>408</x:v>
+        <x:v>407</x:v>
       </x:c>
       <x:c r="D50" s="15" t="s">
-        <x:v>441</x:v>
+        <x:v>440</x:v>
       </x:c>
       <x:c r="E50" s="13"/>
       <x:c r="F50" s="13"/>
@@ -17136,10 +17604,10 @@
         <x:v>13</x:v>
       </x:c>
       <x:c r="C51" s="13" t="s">
-        <x:v>403</x:v>
+        <x:v>402</x:v>
       </x:c>
       <x:c r="D51" s="15" t="s">
-        <x:v>442</x:v>
+        <x:v>441</x:v>
       </x:c>
       <x:c r="E51" s="13"/>
       <x:c r="F51" s="13"/>
@@ -17158,7 +17626,7 @@
         <x:v>82</x:v>
       </x:c>
       <x:c r="D52" s="15" t="s">
-        <x:v>443</x:v>
+        <x:v>442</x:v>
       </x:c>
       <x:c r="E52" s="13"/>
       <x:c r="F52" s="13"/>
@@ -17174,10 +17642,10 @@
         <x:v>13</x:v>
       </x:c>
       <x:c r="C53" s="13" t="s">
-        <x:v>406</x:v>
+        <x:v>405</x:v>
       </x:c>
       <x:c r="D53" s="15" t="s">
-        <x:v>444</x:v>
+        <x:v>443</x:v>
       </x:c>
       <x:c r="E53" s="13"/>
       <x:c r="F53" s="13"/>
@@ -17193,10 +17661,10 @@
         <x:v>13</x:v>
       </x:c>
       <x:c r="C54" s="13" t="s">
-        <x:v>401</x:v>
+        <x:v>400</x:v>
       </x:c>
       <x:c r="D54" s="15" t="s">
-        <x:v>444</x:v>
+        <x:v>443</x:v>
       </x:c>
       <x:c r="E54" s="13"/>
       <x:c r="F54" s="13"/>
@@ -17212,10 +17680,10 @@
         <x:v>13</x:v>
       </x:c>
       <x:c r="C55" s="13" t="s">
-        <x:v>408</x:v>
+        <x:v>407</x:v>
       </x:c>
       <x:c r="D55" s="15" t="s">
-        <x:v>445</x:v>
+        <x:v>444</x:v>
       </x:c>
       <x:c r="E55" s="13"/>
       <x:c r="F55" s="13"/>
@@ -17231,10 +17699,10 @@
         <x:v>359</x:v>
       </x:c>
       <x:c r="C56" s="13" t="s">
-        <x:v>401</x:v>
+        <x:v>400</x:v>
       </x:c>
       <x:c r="D56" s="15" t="s">
-        <x:v>446</x:v>
+        <x:v>445</x:v>
       </x:c>
       <x:c r="E56" s="13"/>
       <x:c r="F56" s="13"/>
@@ -17250,10 +17718,10 @@
         <x:v>359</x:v>
       </x:c>
       <x:c r="C57" s="13" t="s">
-        <x:v>401</x:v>
+        <x:v>400</x:v>
       </x:c>
       <x:c r="D57" s="15" t="s">
-        <x:v>447</x:v>
+        <x:v>446</x:v>
       </x:c>
       <x:c r="E57" s="46"/>
       <x:c r="F57" s="46"/>
@@ -17270,10 +17738,10 @@
         <x:v>359</x:v>
       </x:c>
       <x:c r="C58" s="13" t="s">
-        <x:v>401</x:v>
+        <x:v>400</x:v>
       </x:c>
       <x:c r="D58" s="15" t="s">
-        <x:v>448</x:v>
+        <x:v>447</x:v>
       </x:c>
       <x:c r="E58" s="46"/>
       <x:c r="F58" s="46"/>
@@ -17290,10 +17758,10 @@
         <x:v>359</x:v>
       </x:c>
       <x:c r="C59" s="13" t="s">
-        <x:v>401</x:v>
+        <x:v>400</x:v>
       </x:c>
       <x:c r="D59" s="15" t="s">
-        <x:v>449</x:v>
+        <x:v>448</x:v>
       </x:c>
       <x:c r="E59" s="46"/>
       <x:c r="F59" s="46"/>
@@ -17310,7 +17778,7 @@
         <x:v>95</x:v>
       </x:c>
       <x:c r="D60" s="15" t="s">
-        <x:v>450</x:v>
+        <x:v>449</x:v>
       </x:c>
       <x:c r="E60" s="47">
         <x:v>46277.0</x:v>
@@ -17325,7 +17793,7 @@
         <x:v>103</x:v>
       </x:c>
       <x:c r="I60" s="15" t="s">
-        <x:v>451</x:v>
+        <x:v>450</x:v>
       </x:c>
     </x:row>
     <x:row r="61" ht="48.75" customHeight="1">
@@ -17337,7 +17805,7 @@
         <x:v>95</x:v>
       </x:c>
       <x:c r="D61" s="15" t="s">
-        <x:v>452</x:v>
+        <x:v>451</x:v>
       </x:c>
       <x:c r="E61" s="47">
         <x:v>46277.0</x:v>
@@ -17352,7 +17820,7 @@
         <x:v>113</x:v>
       </x:c>
       <x:c r="I61" s="15" t="s">
-        <x:v>453</x:v>
+        <x:v>452</x:v>
       </x:c>
     </x:row>
     <x:row r="62" ht="48.75" customHeight="1">
@@ -17364,7 +17832,7 @@
         <x:v>95</x:v>
       </x:c>
       <x:c r="D62" s="15" t="s">
-        <x:v>454</x:v>
+        <x:v>453</x:v>
       </x:c>
       <x:c r="E62" s="47">
         <x:v>46277.0</x:v>
@@ -17379,7 +17847,7 @@
         <x:v>103</x:v>
       </x:c>
       <x:c r="I62" s="15" t="s">
-        <x:v>455</x:v>
+        <x:v>454</x:v>
       </x:c>
     </x:row>
     <x:row r="63" ht="48.75" customHeight="1">
@@ -17391,7 +17859,7 @@
         <x:v>95</x:v>
       </x:c>
       <x:c r="D63" s="15" t="s">
-        <x:v>456</x:v>
+        <x:v>455</x:v>
       </x:c>
       <x:c r="E63" s="47">
         <x:v>46277.0</x:v>
@@ -17406,7 +17874,7 @@
         <x:v>113</x:v>
       </x:c>
       <x:c r="I63" s="15" t="s">
-        <x:v>457</x:v>
+        <x:v>456</x:v>
       </x:c>
     </x:row>
     <x:row r="64" ht="48.75" customHeight="1">
@@ -17418,7 +17886,7 @@
         <x:v>95</x:v>
       </x:c>
       <x:c r="D64" s="15" t="s">
-        <x:v>458</x:v>
+        <x:v>457</x:v>
       </x:c>
       <x:c r="E64" s="47">
         <x:v>46277.0</x:v>
@@ -17433,7 +17901,7 @@
         <x:v>103</x:v>
       </x:c>
       <x:c r="I64" s="15" t="s">
-        <x:v>459</x:v>
+        <x:v>458</x:v>
       </x:c>
     </x:row>
     <x:row r="65" ht="48.75" customHeight="1">
@@ -17445,7 +17913,7 @@
         <x:v>95</x:v>
       </x:c>
       <x:c r="D65" s="15" t="s">
-        <x:v>460</x:v>
+        <x:v>459</x:v>
       </x:c>
       <x:c r="E65" s="47">
         <x:v>46277.0</x:v>
@@ -17460,7 +17928,7 @@
         <x:v>113</x:v>
       </x:c>
       <x:c r="I65" s="15" t="s">
-        <x:v>461</x:v>
+        <x:v>460</x:v>
       </x:c>
     </x:row>
     <x:row r="66" ht="48.75" customHeight="1">
@@ -17469,10 +17937,10 @@
         <x:v>13</x:v>
       </x:c>
       <x:c r="C66" s="13" t="s">
+        <x:v>461</x:v>
+      </x:c>
+      <x:c r="D66" s="15" t="s">
         <x:v>462</x:v>
-      </x:c>
-      <x:c r="D66" s="15" t="s">
-        <x:v>463</x:v>
       </x:c>
       <x:c r="E66" s="47">
         <x:v>46277.0</x:v>
@@ -17487,7 +17955,7 @@
         <x:v>113</x:v>
       </x:c>
       <x:c r="I66" s="15" t="s">
-        <x:v>464</x:v>
+        <x:v>463</x:v>
       </x:c>
     </x:row>
     <x:row r="67" ht="48.75" customHeight="1">
@@ -17496,10 +17964,10 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="C67" s="13" t="s">
-        <x:v>462</x:v>
+        <x:v>461</x:v>
       </x:c>
       <x:c r="D67" s="15" t="s">
-        <x:v>465</x:v>
+        <x:v>464</x:v>
       </x:c>
       <x:c r="E67" s="47">
         <x:v>46277.0</x:v>
@@ -17514,7 +17982,7 @@
         <x:v>103</x:v>
       </x:c>
       <x:c r="I67" s="15" t="s">
-        <x:v>466</x:v>
+        <x:v>465</x:v>
       </x:c>
     </x:row>
     <x:row r="68" ht="48.75" customHeight="1">
@@ -17526,7 +17994,7 @@
         <x:v>95</x:v>
       </x:c>
       <x:c r="D68" s="15" t="s">
-        <x:v>467</x:v>
+        <x:v>466</x:v>
       </x:c>
       <x:c r="E68" s="47">
         <x:v>46277.0</x:v>
@@ -17541,7 +18009,7 @@
         <x:v>113</x:v>
       </x:c>
       <x:c r="I68" s="15" t="s">
-        <x:v>468</x:v>
+        <x:v>467</x:v>
       </x:c>
     </x:row>
     <x:row r="69" ht="48.75" customHeight="1">
@@ -17553,7 +18021,7 @@
         <x:v>95</x:v>
       </x:c>
       <x:c r="D69" s="15" t="s">
-        <x:v>469</x:v>
+        <x:v>468</x:v>
       </x:c>
       <x:c r="E69" s="47">
         <x:v>46277.0</x:v>
@@ -17568,7 +18036,7 @@
         <x:v>103</x:v>
       </x:c>
       <x:c r="I69" s="15" t="s">
-        <x:v>470</x:v>
+        <x:v>469</x:v>
       </x:c>
     </x:row>
     <x:row r="70" ht="15.75" customHeight="1">
@@ -17580,10 +18048,10 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="C70" s="3" t="s">
+        <x:v>470</x:v>
+      </x:c>
+      <x:c r="D70" s="48" t="s">
         <x:v>471</x:v>
-      </x:c>
-      <x:c r="D70" s="48" t="s">
-        <x:v>472</x:v>
       </x:c>
       <x:c r="E70" s="49">
         <x:v>46278.0</x:v>
@@ -17598,7 +18066,7 @@
         <x:v>103</x:v>
       </x:c>
       <x:c r="I70" s="4" t="s">
-        <x:v>473</x:v>
+        <x:v>472</x:v>
       </x:c>
     </x:row>
     <x:row r="71" ht="15.75" customHeight="1">
@@ -17610,10 +18078,10 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="C71" s="3" t="s">
-        <x:v>471</x:v>
+        <x:v>470</x:v>
       </x:c>
       <x:c r="D71" s="48" t="s">
-        <x:v>474</x:v>
+        <x:v>473</x:v>
       </x:c>
       <x:c r="E71" s="49">
         <x:v>46278.0</x:v>
@@ -17628,7 +18096,7 @@
         <x:v>113</x:v>
       </x:c>
       <x:c r="I71" s="4" t="s">
-        <x:v>473</x:v>
+        <x:v>472</x:v>
       </x:c>
     </x:row>
     <x:row r="72" ht="15.75" customHeight="1">
@@ -17640,10 +18108,10 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="C72" s="3" t="s">
-        <x:v>471</x:v>
+        <x:v>470</x:v>
       </x:c>
       <x:c r="D72" s="4" t="s">
-        <x:v>475</x:v>
+        <x:v>474</x:v>
       </x:c>
       <x:c r="E72" s="49">
         <x:v>46278.0</x:v>
@@ -17658,7 +18126,7 @@
         <x:v>103</x:v>
       </x:c>
       <x:c r="I72" s="4" t="s">
-        <x:v>473</x:v>
+        <x:v>472</x:v>
       </x:c>
     </x:row>
     <x:row r="73" ht="15.75" customHeight="1">
@@ -17670,10 +18138,10 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="C73" s="3" t="s">
-        <x:v>471</x:v>
+        <x:v>470</x:v>
       </x:c>
       <x:c r="D73" s="4" t="s">
-        <x:v>476</x:v>
+        <x:v>475</x:v>
       </x:c>
       <x:c r="E73" s="49">
         <x:v>46278.0</x:v>
@@ -17688,7 +18156,7 @@
         <x:v>113</x:v>
       </x:c>
       <x:c r="I73" s="4" t="s">
-        <x:v>473</x:v>
+        <x:v>472</x:v>
       </x:c>
     </x:row>
     <x:row r="74" ht="15.75" customHeight="1">
@@ -17700,10 +18168,10 @@
         <x:v>9</x:v>
       </x:c>
       <x:c r="C74" s="3" t="s">
-        <x:v>471</x:v>
+        <x:v>470</x:v>
       </x:c>
       <x:c r="D74" s="4" t="s">
-        <x:v>477</x:v>
+        <x:v>476</x:v>
       </x:c>
       <x:c r="E74" s="49">
         <x:v>46278.0</x:v>
@@ -17718,7 +18186,7 @@
         <x:v>103</x:v>
       </x:c>
       <x:c r="I74" s="4" t="s">
-        <x:v>473</x:v>
+        <x:v>472</x:v>
       </x:c>
     </x:row>
     <x:row r="75" ht="15.75" customHeight="1">
@@ -17730,10 +18198,10 @@
         <x:v>9</x:v>
       </x:c>
       <x:c r="C75" s="3" t="s">
-        <x:v>471</x:v>
+        <x:v>470</x:v>
       </x:c>
       <x:c r="D75" s="4" t="s">
-        <x:v>478</x:v>
+        <x:v>477</x:v>
       </x:c>
       <x:c r="E75" s="49">
         <x:v>46278.0</x:v>
@@ -17748,7 +18216,7 @@
         <x:v>113</x:v>
       </x:c>
       <x:c r="I75" s="4" t="s">
-        <x:v>473</x:v>
+        <x:v>472</x:v>
       </x:c>
     </x:row>
     <x:row r="76" ht="15.75" customHeight="1">
@@ -17760,10 +18228,10 @@
         <x:v>9</x:v>
       </x:c>
       <x:c r="C76" s="3" t="s">
-        <x:v>471</x:v>
+        <x:v>470</x:v>
       </x:c>
       <x:c r="D76" s="50" t="s">
-        <x:v>479</x:v>
+        <x:v>478</x:v>
       </x:c>
       <x:c r="E76" s="49">
         <x:v>46278.0</x:v>
@@ -17778,7 +18246,7 @@
         <x:v>103</x:v>
       </x:c>
       <x:c r="I76" s="4" t="s">
-        <x:v>473</x:v>
+        <x:v>472</x:v>
       </x:c>
     </x:row>
     <x:row r="77" ht="15.75" customHeight="1">
@@ -17790,10 +18258,10 @@
         <x:v>9</x:v>
       </x:c>
       <x:c r="C77" s="3" t="s">
-        <x:v>471</x:v>
+        <x:v>470</x:v>
       </x:c>
       <x:c r="D77" s="50" t="s">
-        <x:v>480</x:v>
+        <x:v>479</x:v>
       </x:c>
       <x:c r="E77" s="49">
         <x:v>46278.0</x:v>
@@ -17808,7 +18276,7 @@
         <x:v>113</x:v>
       </x:c>
       <x:c r="I77" s="4" t="s">
-        <x:v>473</x:v>
+        <x:v>472</x:v>
       </x:c>
     </x:row>
     <x:row r="78" ht="15.75" customHeight="1">
@@ -17820,10 +18288,10 @@
         <x:v>13</x:v>
       </x:c>
       <x:c r="C78" s="3" t="s">
-        <x:v>471</x:v>
+        <x:v>470</x:v>
       </x:c>
       <x:c r="D78" s="50" t="s">
-        <x:v>481</x:v>
+        <x:v>480</x:v>
       </x:c>
       <x:c r="E78" s="49">
         <x:v>46278.0</x:v>
@@ -17838,7 +18306,7 @@
         <x:v>103</x:v>
       </x:c>
       <x:c r="I78" s="4" t="s">
-        <x:v>473</x:v>
+        <x:v>472</x:v>
       </x:c>
     </x:row>
     <x:row r="79" ht="15.75" customHeight="1">
@@ -17850,10 +18318,10 @@
         <x:v>13</x:v>
       </x:c>
       <x:c r="C79" s="3" t="s">
-        <x:v>471</x:v>
+        <x:v>470</x:v>
       </x:c>
       <x:c r="D79" s="50" t="s">
-        <x:v>482</x:v>
+        <x:v>481</x:v>
       </x:c>
       <x:c r="E79" s="49">
         <x:v>46278.0</x:v>
@@ -17868,7 +18336,7 @@
         <x:v>113</x:v>
       </x:c>
       <x:c r="I79" s="4" t="s">
-        <x:v>473</x:v>
+        <x:v>472</x:v>
       </x:c>
     </x:row>
     <x:row r="80" ht="15.75" customHeight="1">
@@ -17880,10 +18348,10 @@
         <x:v>13</x:v>
       </x:c>
       <x:c r="C80" s="3" t="s">
-        <x:v>471</x:v>
+        <x:v>470</x:v>
       </x:c>
       <x:c r="D80" s="50" t="s">
-        <x:v>483</x:v>
+        <x:v>482</x:v>
       </x:c>
       <x:c r="E80" s="49">
         <x:v>46278.0</x:v>
@@ -17898,7 +18366,7 @@
         <x:v>103</x:v>
       </x:c>
       <x:c r="I80" s="4" t="s">
-        <x:v>473</x:v>
+        <x:v>472</x:v>
       </x:c>
     </x:row>
     <x:row r="81" ht="15.75" customHeight="1">
@@ -17910,10 +18378,10 @@
         <x:v>13</x:v>
       </x:c>
       <x:c r="C81" s="3" t="s">
-        <x:v>471</x:v>
+        <x:v>470</x:v>
       </x:c>
       <x:c r="D81" s="50" t="s">
-        <x:v>484</x:v>
+        <x:v>483</x:v>
       </x:c>
       <x:c r="E81" s="49">
         <x:v>46278.0</x:v>
@@ -17928,7 +18396,7 @@
         <x:v>113</x:v>
       </x:c>
       <x:c r="I81" s="4" t="s">
-        <x:v>473</x:v>
+        <x:v>472</x:v>
       </x:c>
     </x:row>
     <x:row r="82" ht="15.75" customHeight="1">
@@ -20470,8 +20938,8 @@
     </x:dataValidation>
   </x:dataValidations>
   <x:hyperlinks>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D70" r:id="R03d9331f54684527"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D71" r:id="R01b6172f4401487c"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D70" r:id="R5a807f2bff424e09"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D71" r:id="Rdee030e70d1b4e68"/>
   </x:hyperlinks>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -20495,325 +20963,325 @@
   <x:sheetData>
     <x:row r="1" ht="33.75" customHeight="1">
       <x:c r="A1" s="51" t="s">
+        <x:v>484</x:v>
+      </x:c>
+      <x:c r="B1" s="51" t="s">
         <x:v>485</x:v>
       </x:c>
-      <x:c r="B1" s="51" t="s">
+      <x:c r="C1" s="51" t="s">
         <x:v>486</x:v>
       </x:c>
-      <x:c r="C1" s="51" t="s">
+      <x:c r="D1" s="51" t="s">
         <x:v>487</x:v>
       </x:c>
-      <x:c r="D1" s="51" t="s">
+      <x:c r="E1" s="51" t="s">
+        <x:v>395</x:v>
+      </x:c>
+      <x:c r="F1" s="51" t="s">
         <x:v>488</x:v>
       </x:c>
-      <x:c r="E1" s="51" t="s">
-        <x:v>396</x:v>
-      </x:c>
-      <x:c r="F1" s="51" t="s">
+      <x:c r="G1" s="51" t="s">
         <x:v>489</x:v>
       </x:c>
-      <x:c r="G1" s="51" t="s">
+      <x:c r="H1" s="51" t="s">
         <x:v>490</x:v>
       </x:c>
-      <x:c r="H1" s="51" t="s">
+      <x:c r="I1" s="51" t="s">
         <x:v>491</x:v>
       </x:c>
-      <x:c r="I1" s="51" t="s">
+      <x:c r="J1" s="51" t="s">
         <x:v>492</x:v>
       </x:c>
-      <x:c r="J1" s="51" t="s">
+      <x:c r="K1" s="51" t="s">
         <x:v>493</x:v>
       </x:c>
-      <x:c r="K1" s="51" t="s">
+      <x:c r="L1" s="51" t="s">
         <x:v>494</x:v>
       </x:c>
-      <x:c r="L1" s="51" t="s">
+      <x:c r="M1" s="51" t="s">
         <x:v>495</x:v>
-      </x:c>
-      <x:c r="M1" s="51" t="s">
-        <x:v>496</x:v>
       </x:c>
     </x:row>
     <x:row r="2">
       <x:c r="A2" s="52" t="s">
+        <x:v>496</x:v>
+      </x:c>
+      <x:c r="B2" s="52" t="s">
         <x:v>497</x:v>
       </x:c>
-      <x:c r="B2" s="52" t="s">
+      <x:c r="C2" s="52" t="s">
         <x:v>498</x:v>
       </x:c>
-      <x:c r="C2" s="52" t="s">
+      <x:c r="D2" s="52" t="s">
         <x:v>499</x:v>
-      </x:c>
-      <x:c r="D2" s="52" t="s">
-        <x:v>500</x:v>
       </x:c>
       <x:c r="E2" s="55">
         <x:v>46278.0</x:v>
       </x:c>
       <x:c r="F2" s="52" t="s">
-        <x:v>501</x:v>
+        <x:v>500</x:v>
       </x:c>
       <x:c r="G2" s="57">
         <x:v>3.4E-5</x:v>
       </x:c>
       <x:c r="H2" s="52" t="s">
+        <x:v>501</x:v>
+      </x:c>
+      <x:c r="I2" s="52" t="s">
         <x:v>502</x:v>
       </x:c>
-      <x:c r="I2" s="52" t="s">
+      <x:c r="J2" s="52" t="s">
         <x:v>503</x:v>
       </x:c>
-      <x:c r="J2" s="52" t="s">
+      <x:c r="K2" s="52" t="s">
         <x:v>504</x:v>
-      </x:c>
-      <x:c r="K2" s="52" t="s">
-        <x:v>505</x:v>
       </x:c>
       <x:c r="L2" s="57" t="n">
         <x:f t="shared" ref="L2:L3" si="1">G2*3600</x:f>
         <x:v>0.1224</x:v>
       </x:c>
       <x:c r="M2" s="52" t="s">
-        <x:v>506</x:v>
+        <x:v>505</x:v>
       </x:c>
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="52" t="s">
-        <x:v>507</x:v>
+        <x:v>506</x:v>
       </x:c>
       <x:c r="B3" s="52" t="s">
+        <x:v>497</x:v>
+      </x:c>
+      <x:c r="C3" s="52" t="s">
         <x:v>498</x:v>
       </x:c>
-      <x:c r="C3" s="52" t="s">
+      <x:c r="D3" s="52" t="s">
         <x:v>499</x:v>
-      </x:c>
-      <x:c r="D3" s="52" t="s">
-        <x:v>500</x:v>
       </x:c>
       <x:c r="E3" s="55">
         <x:v>46278.0</x:v>
       </x:c>
       <x:c r="F3" s="52" t="s">
-        <x:v>508</x:v>
+        <x:v>507</x:v>
       </x:c>
       <x:c r="G3" s="57">
         <x:v>4.0E-6</x:v>
       </x:c>
       <x:c r="H3" s="52" t="s">
+        <x:v>501</x:v>
+      </x:c>
+      <x:c r="I3" s="52" t="s">
         <x:v>502</x:v>
       </x:c>
-      <x:c r="I3" s="52" t="s">
+      <x:c r="J3" s="52" t="s">
         <x:v>503</x:v>
       </x:c>
-      <x:c r="J3" s="52" t="s">
+      <x:c r="K3" s="52" t="s">
         <x:v>504</x:v>
-      </x:c>
-      <x:c r="K3" s="52" t="s">
-        <x:v>505</x:v>
       </x:c>
       <x:c r="L3" s="57">
         <x:f t="shared" si="1"/>
         <x:v>0.0144</x:v>
       </x:c>
       <x:c r="M3" s="52" t="s">
-        <x:v>509</x:v>
+        <x:v>508</x:v>
       </x:c>
     </x:row>
     <x:row r="4">
       <x:c r="A4" s="52" t="s">
-        <x:v>510</x:v>
+        <x:v>509</x:v>
       </x:c>
       <x:c r="B4" s="52" t="s">
+        <x:v>497</x:v>
+      </x:c>
+      <x:c r="C4" s="52" t="s">
         <x:v>498</x:v>
       </x:c>
-      <x:c r="C4" s="52" t="s">
+      <x:c r="D4" s="52" t="s">
         <x:v>499</x:v>
-      </x:c>
-      <x:c r="D4" s="52" t="s">
-        <x:v>500</x:v>
       </x:c>
       <x:c r="E4" s="55">
         <x:v>46278.0</x:v>
       </x:c>
       <x:c r="F4" s="52" t="s">
-        <x:v>511</x:v>
+        <x:v>510</x:v>
       </x:c>
       <x:c r="G4" s="57">
         <x:v>0.4</x:v>
       </x:c>
       <x:c r="H4" s="52" t="s">
+        <x:v>501</x:v>
+      </x:c>
+      <x:c r="I4" s="52" t="s">
         <x:v>502</x:v>
       </x:c>
-      <x:c r="I4" s="52" t="s">
+      <x:c r="J4" s="52" t="s">
         <x:v>503</x:v>
       </x:c>
-      <x:c r="J4" s="52" t="s">
-        <x:v>504</x:v>
-      </x:c>
       <x:c r="K4" s="52" t="s">
-        <x:v>512</x:v>
+        <x:v>511</x:v>
       </x:c>
       <x:c r="L4" s="57" t="n">
         <x:f>G4</x:f>
         <x:v>0.4</x:v>
       </x:c>
       <x:c r="M4" s="52" t="s">
-        <x:v>513</x:v>
+        <x:v>512</x:v>
       </x:c>
     </x:row>
     <x:row r="5">
       <x:c r="A5" s="52" t="s">
+        <x:v>496</x:v>
+      </x:c>
+      <x:c r="B5" s="52" t="s">
         <x:v>497</x:v>
       </x:c>
-      <x:c r="B5" s="52" t="s">
+      <x:c r="C5" s="52" t="s">
         <x:v>498</x:v>
       </x:c>
-      <x:c r="C5" s="52" t="s">
-        <x:v>499</x:v>
-      </x:c>
       <x:c r="D5" s="52" t="s">
-        <x:v>514</x:v>
+        <x:v>513</x:v>
       </x:c>
       <x:c r="E5" s="55">
         <x:v>46278.0</x:v>
       </x:c>
       <x:c r="F5" s="52" t="s">
-        <x:v>501</x:v>
+        <x:v>500</x:v>
       </x:c>
       <x:c r="G5" s="57">
         <x:v>2.4E-5</x:v>
       </x:c>
       <x:c r="H5" s="52" t="s">
-        <x:v>502</x:v>
+        <x:v>501</x:v>
       </x:c>
       <x:c r="I5" s="52" t="s">
+        <x:v>514</x:v>
+      </x:c>
+      <x:c r="J5" s="52" t="s">
         <x:v>515</x:v>
       </x:c>
-      <x:c r="J5" s="52" t="s">
-        <x:v>516</x:v>
-      </x:c>
       <x:c r="K5" s="52" t="s">
-        <x:v>505</x:v>
+        <x:v>504</x:v>
       </x:c>
       <x:c r="L5" s="57" t="n">
         <x:f t="shared" ref="L5:L6" si="2">G5*3600</x:f>
         <x:v>0.0864</x:v>
       </x:c>
       <x:c r="M5" s="52" t="s">
-        <x:v>506</x:v>
+        <x:v>505</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
       <x:c r="A6" s="52" t="s">
-        <x:v>507</x:v>
+        <x:v>506</x:v>
       </x:c>
       <x:c r="B6" s="52" t="s">
+        <x:v>497</x:v>
+      </x:c>
+      <x:c r="C6" s="52" t="s">
         <x:v>498</x:v>
       </x:c>
-      <x:c r="C6" s="52" t="s">
-        <x:v>499</x:v>
-      </x:c>
       <x:c r="D6" s="52" t="s">
-        <x:v>514</x:v>
+        <x:v>513</x:v>
       </x:c>
       <x:c r="E6" s="55">
         <x:v>46278.0</x:v>
       </x:c>
       <x:c r="F6" s="52" t="s">
-        <x:v>508</x:v>
+        <x:v>507</x:v>
       </x:c>
       <x:c r="G6" s="57">
         <x:v>3.0E-6</x:v>
       </x:c>
       <x:c r="H6" s="52" t="s">
-        <x:v>502</x:v>
+        <x:v>501</x:v>
       </x:c>
       <x:c r="I6" s="52" t="s">
+        <x:v>514</x:v>
+      </x:c>
+      <x:c r="J6" s="52" t="s">
         <x:v>515</x:v>
       </x:c>
-      <x:c r="J6" s="52" t="s">
-        <x:v>516</x:v>
-      </x:c>
       <x:c r="K6" s="52" t="s">
-        <x:v>505</x:v>
+        <x:v>504</x:v>
       </x:c>
       <x:c r="L6" s="57">
         <x:f t="shared" si="2"/>
         <x:v>0.0108</x:v>
       </x:c>
       <x:c r="M6" s="52" t="s">
-        <x:v>509</x:v>
+        <x:v>508</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
       <x:c r="A7" s="52" t="s">
-        <x:v>510</x:v>
+        <x:v>509</x:v>
       </x:c>
       <x:c r="B7" s="52" t="s">
+        <x:v>497</x:v>
+      </x:c>
+      <x:c r="C7" s="52" t="s">
         <x:v>498</x:v>
       </x:c>
-      <x:c r="C7" s="52" t="s">
-        <x:v>499</x:v>
-      </x:c>
       <x:c r="D7" s="52" t="s">
-        <x:v>514</x:v>
+        <x:v>513</x:v>
       </x:c>
       <x:c r="E7" s="55">
         <x:v>46278.0</x:v>
       </x:c>
       <x:c r="F7" s="52" t="s">
-        <x:v>511</x:v>
+        <x:v>510</x:v>
       </x:c>
       <x:c r="G7" s="57">
         <x:v>0.4</x:v>
       </x:c>
       <x:c r="H7" s="52" t="s">
-        <x:v>502</x:v>
+        <x:v>501</x:v>
       </x:c>
       <x:c r="I7" s="52" t="s">
+        <x:v>514</x:v>
+      </x:c>
+      <x:c r="J7" s="52" t="s">
         <x:v>515</x:v>
       </x:c>
-      <x:c r="J7" s="52" t="s">
-        <x:v>516</x:v>
-      </x:c>
       <x:c r="K7" s="52" t="s">
-        <x:v>512</x:v>
+        <x:v>511</x:v>
       </x:c>
       <x:c r="L7" s="57" t="n">
         <x:f>G7</x:f>
         <x:v>0.4</x:v>
       </x:c>
       <x:c r="M7" s="52" t="s">
-        <x:v>513</x:v>
+        <x:v>512</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
       <x:c r="A8" s="52" t="s">
+        <x:v>516</x:v>
+      </x:c>
+      <x:c r="B8" s="52" t="s">
         <x:v>517</x:v>
       </x:c>
-      <x:c r="B8" s="52" t="s">
+      <x:c r="C8" s="52" t="s">
+        <x:v>498</x:v>
+      </x:c>
+      <x:c r="D8" s="52" t="s">
         <x:v>518</x:v>
-      </x:c>
-      <x:c r="C8" s="52" t="s">
-        <x:v>499</x:v>
-      </x:c>
-      <x:c r="D8" s="52" t="s">
-        <x:v>519</x:v>
       </x:c>
       <x:c r="E8" s="55">
         <x:v>46278.0</x:v>
       </x:c>
       <x:c r="F8" s="52" t="s">
-        <x:v>520</x:v>
+        <x:v>519</x:v>
       </x:c>
       <x:c r="G8" s="57"/>
       <x:c r="H8" s="52" t="s">
-        <x:v>521</x:v>
+        <x:v>520</x:v>
       </x:c>
       <x:c r="I8" s="52" t="s">
         <x:v>152</x:v>
       </x:c>
       <x:c r="J8" s="52" t="s">
-        <x:v>522</x:v>
+        <x:v>521</x:v>
       </x:c>
       <x:c r="K8" s="52"/>
       <x:c r="L8" s="57"/>
@@ -21638,149 +22106,467 @@
         <x:v>USD/licencia</x:v>
       </x:c>
     </x:row>
-    <x:row r="30" ht="15.75" customHeight="1">
-      <x:c r="A30" s="4"/>
-      <x:c r="B30" s="4"/>
-      <x:c r="C30" s="4"/>
-      <x:c r="D30" s="4"/>
-      <x:c r="E30" s="49"/>
-      <x:c r="F30" s="4"/>
-      <x:c r="G30" s="4"/>
-      <x:c r="H30" s="4"/>
-      <x:c r="I30" s="4"/>
-      <x:c r="J30" s="4"/>
-    </x:row>
-    <x:row r="31" ht="15.75" customHeight="1">
-      <x:c r="A31" s="4"/>
-      <x:c r="B31" s="4"/>
-      <x:c r="C31" s="4"/>
-      <x:c r="D31" s="4"/>
-      <x:c r="E31" s="49"/>
-      <x:c r="F31" s="4"/>
-      <x:c r="G31" s="4"/>
-      <x:c r="H31" s="4"/>
-      <x:c r="I31" s="4"/>
-      <x:c r="J31" s="4"/>
-    </x:row>
-    <x:row r="32" ht="15.75" customHeight="1">
-      <x:c r="A32" s="4"/>
-      <x:c r="B32" s="4"/>
-      <x:c r="C32" s="4"/>
-      <x:c r="D32" s="4"/>
-      <x:c r="E32" s="49"/>
-      <x:c r="F32" s="4"/>
-      <x:c r="G32" s="4"/>
-      <x:c r="H32" s="4"/>
-      <x:c r="I32" s="4"/>
-      <x:c r="J32" s="4"/>
-    </x:row>
-    <x:row r="33" ht="15.75" customHeight="1">
-      <x:c r="A33" s="4"/>
-      <x:c r="B33" s="4"/>
-      <x:c r="C33" s="4"/>
-      <x:c r="D33" s="4"/>
-      <x:c r="E33" s="49"/>
-      <x:c r="F33" s="4"/>
-      <x:c r="G33" s="4"/>
-      <x:c r="H33" s="4"/>
-      <x:c r="I33" s="4"/>
-      <x:c r="J33" s="4"/>
-    </x:row>
-    <x:row r="34" ht="15.75" customHeight="1">
-      <x:c r="A34" s="4"/>
-      <x:c r="B34" s="4"/>
-      <x:c r="C34" s="4"/>
-      <x:c r="D34" s="4"/>
-      <x:c r="E34" s="49"/>
-      <x:c r="F34" s="4"/>
-      <x:c r="G34" s="4"/>
-      <x:c r="H34" s="4"/>
-      <x:c r="I34" s="4"/>
-      <x:c r="J34" s="4"/>
-    </x:row>
-    <x:row r="35" ht="15.75" customHeight="1">
-      <x:c r="A35" s="4"/>
-      <x:c r="B35" s="4"/>
-      <x:c r="C35" s="4"/>
-      <x:c r="D35" s="4"/>
-      <x:c r="E35" s="49"/>
-      <x:c r="F35" s="4"/>
-      <x:c r="G35" s="4"/>
-      <x:c r="H35" s="4"/>
-      <x:c r="I35" s="4"/>
-      <x:c r="J35" s="4"/>
-    </x:row>
-    <x:row r="36" ht="15.75" customHeight="1">
-      <x:c r="A36" s="4"/>
-      <x:c r="B36" s="4"/>
-      <x:c r="C36" s="4"/>
-      <x:c r="D36" s="4"/>
-      <x:c r="E36" s="49"/>
-      <x:c r="F36" s="4"/>
-      <x:c r="G36" s="4"/>
-      <x:c r="H36" s="4"/>
-      <x:c r="I36" s="4"/>
-      <x:c r="J36" s="4"/>
-    </x:row>
-    <x:row r="37" ht="15.75" customHeight="1">
-      <x:c r="A37" s="4"/>
-      <x:c r="B37" s="4"/>
-      <x:c r="C37" s="4"/>
-      <x:c r="D37" s="4"/>
-      <x:c r="E37" s="49"/>
-      <x:c r="F37" s="4"/>
-      <x:c r="G37" s="4"/>
-      <x:c r="H37" s="4"/>
-      <x:c r="I37" s="4"/>
-      <x:c r="J37" s="4"/>
-    </x:row>
-    <x:row r="38" ht="15.75" customHeight="1">
-      <x:c r="A38" s="4"/>
-      <x:c r="B38" s="4"/>
-      <x:c r="C38" s="4"/>
-      <x:c r="D38" s="4"/>
-      <x:c r="E38" s="49"/>
-      <x:c r="F38" s="4"/>
-      <x:c r="G38" s="4"/>
-      <x:c r="H38" s="4"/>
-      <x:c r="I38" s="4"/>
-      <x:c r="J38" s="4"/>
-    </x:row>
-    <x:row r="39" ht="15.75" customHeight="1">
-      <x:c r="A39" s="4"/>
-      <x:c r="B39" s="4"/>
-      <x:c r="C39" s="4"/>
-      <x:c r="D39" s="4"/>
-      <x:c r="E39" s="49"/>
-      <x:c r="F39" s="4"/>
-      <x:c r="G39" s="4"/>
-      <x:c r="H39" s="4"/>
-      <x:c r="I39" s="4"/>
-      <x:c r="J39" s="4"/>
-    </x:row>
-    <x:row r="40" ht="15.75" customHeight="1">
-      <x:c r="A40" s="4"/>
-      <x:c r="B40" s="4"/>
-      <x:c r="C40" s="4"/>
-      <x:c r="D40" s="4"/>
-      <x:c r="E40" s="49"/>
-      <x:c r="F40" s="4"/>
-      <x:c r="G40" s="4"/>
-      <x:c r="H40" s="4"/>
-      <x:c r="I40" s="4"/>
-      <x:c r="J40" s="4"/>
-    </x:row>
-    <x:row r="41" ht="15.75" customHeight="1">
-      <x:c r="A41" s="4"/>
-      <x:c r="B41" s="4"/>
-      <x:c r="C41" s="4"/>
-      <x:c r="D41" s="4"/>
-      <x:c r="E41" s="49"/>
-      <x:c r="F41" s="4"/>
-      <x:c r="G41" s="4"/>
-      <x:c r="H41" s="4"/>
-      <x:c r="I41" s="4"/>
-      <x:c r="J41" s="4"/>
+    <x:row r="30" ht="34" customHeight="1">
+      <x:c r="A30" s="61" t="str">
+        <x:v>Azure Database for PostgreSQL Flexible Server - General Purpose Dsv3 (precio por vCore-hora; base 2 vCores)</x:v>
+      </x:c>
+      <x:c r="B30" s="61" t="str">
+        <x:v>Microsoft Azure</x:v>
+      </x:c>
+      <x:c r="C30" s="61" t="str">
+        <x:v>USD</x:v>
+      </x:c>
+      <x:c r="D30" s="61" t="str">
+        <x:v>Chile Central</x:v>
+      </x:c>
+      <x:c r="E30" s="56" t="n">
+        <x:v>46280</x:v>
+      </x:c>
+      <x:c r="F30" s="61" t="str">
+        <x:v>vCore-hora</x:v>
+      </x:c>
+      <x:c r="G30" s="61" t="n">
+        <x:v>0.1197</x:v>
+      </x:c>
+      <x:c r="H30" s="61" t="str">
+        <x:v>Precio público / regla oficial</x:v>
+      </x:c>
+      <x:c r="I30" s="61" t="str">
+        <x:v>https://learn.microsoft.com/en-us/azure/postgresql/compute-storage/concepts-compute</x:v>
+      </x:c>
+      <x:c r="J30" s="61" t="str">
+        <x:v>General Purpose mínimo 2 vCores; tarifa unitaria por vCore-hora</x:v>
+      </x:c>
+      <x:c r="K30" s="61" t="str">
+        <x:v>Precio × 2 vCores × horas</x:v>
+      </x:c>
+      <x:c r="L30" t="n">
+        <x:f>G30</x:f>
+        <x:v>0.1197</x:v>
+      </x:c>
+      <x:c r="M30" t="str">
+        <x:v>USD/vCore-hora</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="31" ht="34" customHeight="1">
+      <x:c r="A31" s="61" t="str">
+        <x:v>Azure Database for PostgreSQL Flexible Server - Premium SSD v2 Storage</x:v>
+      </x:c>
+      <x:c r="B31" s="61" t="str">
+        <x:v>Microsoft Azure</x:v>
+      </x:c>
+      <x:c r="C31" s="61" t="str">
+        <x:v>USD</x:v>
+      </x:c>
+      <x:c r="D31" s="61" t="str">
+        <x:v>Chile Central</x:v>
+      </x:c>
+      <x:c r="E31" s="56" t="n">
+        <x:v>46280</x:v>
+      </x:c>
+      <x:c r="F31" s="61" t="str">
+        <x:v>GiB-mes</x:v>
+      </x:c>
+      <x:c r="G31" s="61" t="n">
+        <x:v>0.161</x:v>
+      </x:c>
+      <x:c r="H31" s="61" t="str">
+        <x:v>Precio de lista publico</x:v>
+      </x:c>
+      <x:c r="I31" s="61" t="str">
+        <x:v>https://prices.azure.com/api/retail/prices?%24filter=serviceName%20eq%20'Azure%20Database%20for%20PostgreSQL'%20and%20armRegionName%20eq%20'chilecentral'&amp;%24top=100</x:v>
+      </x:c>
+      <x:c r="J31" s="61" t="str">
+        <x:v>effectiveStartDate=2025-04-01; almacenamiento de datos</x:v>
+      </x:c>
+      <x:c r="K31" s="61" t="str">
+        <x:v>Precio API por GiB/mes</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="32" ht="34" customHeight="1">
+      <x:c r="A32" s="61" t="str">
+        <x:v>Azure Blob Storage - General Block Blob v2 Hot LRS</x:v>
+      </x:c>
+      <x:c r="B32" s="61" t="str">
+        <x:v>Microsoft Azure</x:v>
+      </x:c>
+      <x:c r="C32" s="61" t="str">
+        <x:v>USD</x:v>
+      </x:c>
+      <x:c r="D32" s="61" t="str">
+        <x:v>Chile Central</x:v>
+      </x:c>
+      <x:c r="E32" s="56" t="n">
+        <x:v>46280</x:v>
+      </x:c>
+      <x:c r="F32" s="61" t="str">
+        <x:v>GB-mes</x:v>
+      </x:c>
+      <x:c r="G32" s="61" t="n">
+        <x:v>0.02576</x:v>
+      </x:c>
+      <x:c r="H32" s="61" t="str">
+        <x:v>Precio de lista publico; primer tramo</x:v>
+      </x:c>
+      <x:c r="I32" s="61" t="str">
+        <x:v>https://prices.azure.com/api/retail/prices?%24filter=serviceName%20eq%20'Storage'%20and%20armRegionName%20eq%20'chilecentral'&amp;%24top=100</x:v>
+      </x:c>
+      <x:c r="J32" s="61" t="str">
+        <x:v>effectiveStartDate=2025-04-01; Hot LRS Data Stored</x:v>
+      </x:c>
+      <x:c r="K32" s="61" t="str">
+        <x:v>Precio API por GB/mes</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="33" ht="34" customHeight="1">
+      <x:c r="A33" s="61" t="str">
+        <x:v>Azure Bandwidth - Internet Egress Premium Global Network (South America)</x:v>
+      </x:c>
+      <x:c r="B33" s="61" t="str">
+        <x:v>Microsoft Azure</x:v>
+      </x:c>
+      <x:c r="C33" s="61" t="str">
+        <x:v>USD</x:v>
+      </x:c>
+      <x:c r="D33" s="61" t="str">
+        <x:v>Chile Central</x:v>
+      </x:c>
+      <x:c r="E33" s="56" t="n">
+        <x:v>46280</x:v>
+      </x:c>
+      <x:c r="F33" s="61" t="str">
+        <x:v>GB</x:v>
+      </x:c>
+      <x:c r="G33" s="61" t="n">
+        <x:v>0.181</x:v>
+      </x:c>
+      <x:c r="H33" s="61" t="str">
+        <x:v>Precio público / regla oficial</x:v>
+      </x:c>
+      <x:c r="I33" s="61" t="str">
+        <x:v>https://azure.microsoft.com/en-us/pricing/details/bandwidth/</x:v>
+      </x:c>
+      <x:c r="J33" s="61" t="str">
+        <x:v>Primeros 100 GB/mes gratis; próximos 10 TB</x:v>
+      </x:c>
+      <x:c r="K33" s="61" t="str">
+        <x:v>MAX(GB-100,0) × precio</x:v>
+      </x:c>
+      <x:c r="L33" t="n">
+        <x:f>G33</x:f>
+        <x:v>0.181</x:v>
+      </x:c>
+      <x:c r="M33" t="str">
+        <x:v>USD/GB</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="34" ht="34" customHeight="1">
+      <x:c r="A34" s="61" t="str">
+        <x:v>Azure Monitor - Basic Logs Data Ingestion</x:v>
+      </x:c>
+      <x:c r="B34" s="61" t="str">
+        <x:v>Microsoft Azure</x:v>
+      </x:c>
+      <x:c r="C34" s="61" t="str">
+        <x:v>USD</x:v>
+      </x:c>
+      <x:c r="D34" s="61" t="str">
+        <x:v>Chile Central</x:v>
+      </x:c>
+      <x:c r="E34" s="56" t="n">
+        <x:v>46280</x:v>
+      </x:c>
+      <x:c r="F34" s="61" t="str">
+        <x:v>GB</x:v>
+      </x:c>
+      <x:c r="G34" s="61" t="n">
+        <x:v>0.7</x:v>
+      </x:c>
+      <x:c r="H34" s="61" t="str">
+        <x:v>Precio de lista publico</x:v>
+      </x:c>
+      <x:c r="I34" s="61" t="str">
+        <x:v>https://prices.azure.com/api/retail/prices?%24filter=serviceName%20eq%20'Azure%20Monitor'%20and%20armRegionName%20eq%20'chilecentral'&amp;%24top=100</x:v>
+      </x:c>
+      <x:c r="J34" s="61" t="str">
+        <x:v>effectiveStartDate=2025-04-01; Basic Logs</x:v>
+      </x:c>
+      <x:c r="K34" s="61" t="str">
+        <x:v>Precio API por GB ingerido</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="35" ht="34" customHeight="1">
+      <x:c r="A35" s="61" t="str">
+        <x:v>Azure PostgreSQL - Automated Backup Storage Overage</x:v>
+      </x:c>
+      <x:c r="B35" s="61" t="str">
+        <x:v>Microsoft Azure</x:v>
+      </x:c>
+      <x:c r="C35" s="61" t="str">
+        <x:v>USD</x:v>
+      </x:c>
+      <x:c r="D35" s="61" t="str">
+        <x:v>Chile Central</x:v>
+      </x:c>
+      <x:c r="E35" s="56" t="n">
+        <x:v>46280</x:v>
+      </x:c>
+      <x:c r="F35" s="61" t="str">
+        <x:v>instancia-mes</x:v>
+      </x:c>
+      <x:c r="G35" s="61" t="n">
+        <x:v>0.095</x:v>
+      </x:c>
+      <x:c r="H35" s="61" t="str">
+        <x:v>Precio público / regla oficial</x:v>
+      </x:c>
+      <x:c r="I35" s="61" t="str">
+        <x:v>https://azure.microsoft.com/en-us/pricing/details/postgresql/flexible-server/</x:v>
+      </x:c>
+      <x:c r="J35" s="61" t="str">
+        <x:v>Sin cargo hasta 100% del storage provisionado; base 0 GiB excedente</x:v>
+      </x:c>
+      <x:c r="K35" s="61" t="str">
+        <x:v>GiB excedente × precio</x:v>
+      </x:c>
+      <x:c r="L35" t="n">
+        <x:f>G35</x:f>
+        <x:v>0.095</x:v>
+      </x:c>
+      <x:c r="M35" t="str">
+        <x:v>USD/GiB-mes</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="36" ht="34" customHeight="1">
+      <x:c r="A36" s="61" t="str">
+        <x:v>Azure Database for PostgreSQL Flexible Server - General Purpose Dsv3 (precio por vCore-hora; base 2 vCores)</x:v>
+      </x:c>
+      <x:c r="B36" s="61" t="str">
+        <x:v>Microsoft Azure</x:v>
+      </x:c>
+      <x:c r="C36" s="61" t="str">
+        <x:v>USD</x:v>
+      </x:c>
+      <x:c r="D36" s="61" t="str">
+        <x:v>East US</x:v>
+      </x:c>
+      <x:c r="E36" s="56" t="n">
+        <x:v>46280</x:v>
+      </x:c>
+      <x:c r="F36" s="61" t="str">
+        <x:v>vCore-hora</x:v>
+      </x:c>
+      <x:c r="G36" s="61" t="n">
+        <x:v>0.0855</x:v>
+      </x:c>
+      <x:c r="H36" s="61" t="str">
+        <x:v>Precio público / regla oficial</x:v>
+      </x:c>
+      <x:c r="I36" s="61" t="str">
+        <x:v>https://learn.microsoft.com/en-us/azure/postgresql/compute-storage/concepts-compute</x:v>
+      </x:c>
+      <x:c r="J36" s="61" t="str">
+        <x:v>General Purpose mínimo 2 vCores; tarifa unitaria por vCore-hora</x:v>
+      </x:c>
+      <x:c r="K36" s="61" t="str">
+        <x:v>Precio × 2 vCores × horas</x:v>
+      </x:c>
+      <x:c r="L36" t="n">
+        <x:f>G36</x:f>
+        <x:v>0.0855</x:v>
+      </x:c>
+      <x:c r="M36" t="str">
+        <x:v>USD/vCore-hora</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="37" ht="34" customHeight="1">
+      <x:c r="A37" s="61" t="str">
+        <x:v>Azure Database for PostgreSQL Flexible Server - Premium SSD v2 Storage</x:v>
+      </x:c>
+      <x:c r="B37" s="61" t="str">
+        <x:v>Microsoft Azure</x:v>
+      </x:c>
+      <x:c r="C37" s="61" t="str">
+        <x:v>USD</x:v>
+      </x:c>
+      <x:c r="D37" s="61" t="str">
+        <x:v>East US</x:v>
+      </x:c>
+      <x:c r="E37" s="56" t="n">
+        <x:v>46280</x:v>
+      </x:c>
+      <x:c r="F37" s="61" t="str">
+        <x:v>GiB-mes</x:v>
+      </x:c>
+      <x:c r="G37" s="61" t="n">
+        <x:v>0.115</x:v>
+      </x:c>
+      <x:c r="H37" s="61" t="str">
+        <x:v>Precio de lista publico</x:v>
+      </x:c>
+      <x:c r="I37" s="61" t="str">
+        <x:v>https://prices.azure.com/api/retail/prices?%24filter=serviceName%20eq%20'Azure%20Database%20for%20PostgreSQL'%20and%20armRegionName%20eq%20'eastus'&amp;%24top=100</x:v>
+      </x:c>
+      <x:c r="J37" s="61" t="str">
+        <x:v>effectiveStartDate=2023-10-01; almacenamiento de datos</x:v>
+      </x:c>
+      <x:c r="K37" s="61" t="str">
+        <x:v>Precio API por GiB/mes</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="38" ht="34" customHeight="1">
+      <x:c r="A38" s="61" t="str">
+        <x:v>Azure Blob Storage - General Block Blob v2 Hot LRS</x:v>
+      </x:c>
+      <x:c r="B38" s="61" t="str">
+        <x:v>Microsoft Azure</x:v>
+      </x:c>
+      <x:c r="C38" s="61" t="str">
+        <x:v>USD</x:v>
+      </x:c>
+      <x:c r="D38" s="61" t="str">
+        <x:v>East US</x:v>
+      </x:c>
+      <x:c r="E38" s="56" t="n">
+        <x:v>46280</x:v>
+      </x:c>
+      <x:c r="F38" s="61" t="str">
+        <x:v>GB-mes</x:v>
+      </x:c>
+      <x:c r="G38" s="61" t="n">
+        <x:v>0.0208</x:v>
+      </x:c>
+      <x:c r="H38" s="61" t="str">
+        <x:v>Precio de lista publico; primer tramo</x:v>
+      </x:c>
+      <x:c r="I38" s="61" t="str">
+        <x:v>https://prices.azure.com/api/retail/prices?%24filter=serviceName%20eq%20'Storage'%20and%20armRegionName%20eq%20'eastus'&amp;%24top=100</x:v>
+      </x:c>
+      <x:c r="J38" s="61" t="str">
+        <x:v>effectiveStartDate=2025-04-01; Hot LRS Data Stored</x:v>
+      </x:c>
+      <x:c r="K38" s="61" t="str">
+        <x:v>Precio API por GB/mes</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="39" ht="34" customHeight="1">
+      <x:c r="A39" s="61" t="str">
+        <x:v>Azure Bandwidth - Internet Egress Premium Global Network (North America)</x:v>
+      </x:c>
+      <x:c r="B39" s="61" t="str">
+        <x:v>Microsoft Azure</x:v>
+      </x:c>
+      <x:c r="C39" s="61" t="str">
+        <x:v>USD</x:v>
+      </x:c>
+      <x:c r="D39" s="61" t="str">
+        <x:v>East US</x:v>
+      </x:c>
+      <x:c r="E39" s="56" t="n">
+        <x:v>46280</x:v>
+      </x:c>
+      <x:c r="F39" s="61" t="str">
+        <x:v>GB</x:v>
+      </x:c>
+      <x:c r="G39" s="61" t="n">
+        <x:v>0.087</x:v>
+      </x:c>
+      <x:c r="H39" s="61" t="str">
+        <x:v>Precio público / regla oficial</x:v>
+      </x:c>
+      <x:c r="I39" s="61" t="str">
+        <x:v>https://azure.microsoft.com/en-us/pricing/details/bandwidth/</x:v>
+      </x:c>
+      <x:c r="J39" s="61" t="str">
+        <x:v>Primeros 100 GB/mes gratis; próximos 10 TB</x:v>
+      </x:c>
+      <x:c r="K39" s="61" t="str">
+        <x:v>MAX(GB-100,0) × precio</x:v>
+      </x:c>
+      <x:c r="L39" t="n">
+        <x:f>G39</x:f>
+        <x:v>0.087</x:v>
+      </x:c>
+      <x:c r="M39" t="str">
+        <x:v>USD/GB</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="40" ht="34" customHeight="1">
+      <x:c r="A40" s="61" t="str">
+        <x:v>Azure Monitor - Basic Logs Data Ingestion</x:v>
+      </x:c>
+      <x:c r="B40" s="61" t="str">
+        <x:v>Microsoft Azure</x:v>
+      </x:c>
+      <x:c r="C40" s="61" t="str">
+        <x:v>USD</x:v>
+      </x:c>
+      <x:c r="D40" s="61" t="str">
+        <x:v>East US</x:v>
+      </x:c>
+      <x:c r="E40" s="56" t="n">
+        <x:v>46280</x:v>
+      </x:c>
+      <x:c r="F40" s="61" t="str">
+        <x:v>GB</x:v>
+      </x:c>
+      <x:c r="G40" s="61" t="n">
+        <x:v>0.5</x:v>
+      </x:c>
+      <x:c r="H40" s="61" t="str">
+        <x:v>Precio de lista publico</x:v>
+      </x:c>
+      <x:c r="I40" s="61" t="str">
+        <x:v>https://prices.azure.com/api/retail/prices?%24filter=serviceName%20eq%20'Azure%20Monitor'%20and%20armRegionName%20eq%20'eastus'&amp;%24top=100</x:v>
+      </x:c>
+      <x:c r="J40" s="61" t="str">
+        <x:v>effectiveStartDate=2022-10-01; Basic Logs</x:v>
+      </x:c>
+      <x:c r="K40" s="61" t="str">
+        <x:v>Precio API por GB ingerido</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="41" ht="34" customHeight="1">
+      <x:c r="A41" s="61" t="str">
+        <x:v>Azure PostgreSQL - Automated Backup Storage Overage</x:v>
+      </x:c>
+      <x:c r="B41" s="61" t="str">
+        <x:v>Microsoft Azure</x:v>
+      </x:c>
+      <x:c r="C41" s="61" t="str">
+        <x:v>USD</x:v>
+      </x:c>
+      <x:c r="D41" s="61" t="str">
+        <x:v>East US</x:v>
+      </x:c>
+      <x:c r="E41" s="56" t="n">
+        <x:v>46280</x:v>
+      </x:c>
+      <x:c r="F41" s="61" t="str">
+        <x:v>instancia-mes</x:v>
+      </x:c>
+      <x:c r="G41" s="61" t="n">
+        <x:v>0.095</x:v>
+      </x:c>
+      <x:c r="H41" s="61" t="str">
+        <x:v>Precio público / regla oficial</x:v>
+      </x:c>
+      <x:c r="I41" s="61" t="str">
+        <x:v>https://azure.microsoft.com/en-us/pricing/details/postgresql/flexible-server/</x:v>
+      </x:c>
+      <x:c r="J41" s="61" t="str">
+        <x:v>Sin cargo hasta 100% del storage provisionado; base 0 GiB excedente</x:v>
+      </x:c>
+      <x:c r="K41" s="61" t="str">
+        <x:v>GiB excedente × precio</x:v>
+      </x:c>
+      <x:c r="L41" t="n">
+        <x:f>G41</x:f>
+        <x:v>0.095</x:v>
+      </x:c>
+      <x:c r="M41" t="str">
+        <x:v>USD/GiB-mes</x:v>
+      </x:c>
     </x:row>
     <x:row r="42" ht="15.75" customHeight="1">
       <x:c r="A42" s="4"/>
@@ -23411,57 +24197,57 @@
   <x:sheetData>
     <x:row r="1" ht="33.75" customHeight="1">
       <x:c r="A1" s="34" t="s">
+        <x:v>522</x:v>
+      </x:c>
+      <x:c r="B1" s="34" t="s">
         <x:v>523</x:v>
       </x:c>
-      <x:c r="B1" s="34" t="s">
+      <x:c r="C1" s="34" t="s">
+        <x:v>485</x:v>
+      </x:c>
+      <x:c r="D1" s="34" t="s">
         <x:v>524</x:v>
       </x:c>
-      <x:c r="C1" s="34" t="s">
-        <x:v>486</x:v>
-      </x:c>
-      <x:c r="D1" s="34" t="s">
+      <x:c r="E1" s="34" t="s">
+        <x:v>487</x:v>
+      </x:c>
+      <x:c r="F1" s="34" t="s">
         <x:v>525</x:v>
       </x:c>
-      <x:c r="E1" s="34" t="s">
-        <x:v>488</x:v>
-      </x:c>
-      <x:c r="F1" s="34" t="s">
+      <x:c r="G1" s="34" t="s">
         <x:v>526</x:v>
-      </x:c>
-      <x:c r="G1" s="34" t="s">
-        <x:v>527</x:v>
       </x:c>
       <x:c r="H1" s="34" t="s">
         <x:v>78</x:v>
       </x:c>
       <x:c r="I1" s="34" t="s">
-        <x:v>528</x:v>
+        <x:v>527</x:v>
       </x:c>
     </x:row>
     <x:row r="2">
       <x:c r="A2" s="4" t="s">
+        <x:v>528</x:v>
+      </x:c>
+      <x:c r="B2" s="4" t="s">
+        <x:v>516</x:v>
+      </x:c>
+      <x:c r="C2" s="4" t="s">
+        <x:v>517</x:v>
+      </x:c>
+      <x:c r="D2" s="4" t="s">
         <x:v>529</x:v>
       </x:c>
-      <x:c r="B2" s="4" t="s">
-        <x:v>517</x:v>
-      </x:c>
-      <x:c r="C2" s="4" t="s">
+      <x:c r="E2" s="4" t="s">
         <x:v>518</x:v>
       </x:c>
-      <x:c r="D2" s="4" t="s">
+      <x:c r="F2" s="4" t="s">
         <x:v>530</x:v>
-      </x:c>
-      <x:c r="E2" s="4" t="s">
-        <x:v>519</x:v>
-      </x:c>
-      <x:c r="F2" s="4" t="s">
-        <x:v>531</x:v>
       </x:c>
       <x:c r="G2" s="4" t="s">
         <x:v>152</x:v>
       </x:c>
       <x:c r="H2" s="4" t="s">
-        <x:v>532</x:v>
+        <x:v>531</x:v>
       </x:c>
       <x:c r="I2" s="49">
         <x:v>46277.0</x:v>
@@ -23469,28 +24255,28 @@
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="4" t="s">
+        <x:v>528</x:v>
+      </x:c>
+      <x:c r="B3" s="4" t="s">
+        <x:v>532</x:v>
+      </x:c>
+      <x:c r="C3" s="4" t="s">
+        <x:v>497</x:v>
+      </x:c>
+      <x:c r="D3" s="4" t="s">
         <x:v>529</x:v>
       </x:c>
-      <x:c r="B3" s="4" t="s">
+      <x:c r="E3" s="4" t="s">
+        <x:v>499</x:v>
+      </x:c>
+      <x:c r="F3" s="4" t="s">
         <x:v>533</x:v>
-      </x:c>
-      <x:c r="C3" s="4" t="s">
-        <x:v>498</x:v>
-      </x:c>
-      <x:c r="D3" s="4" t="s">
-        <x:v>530</x:v>
-      </x:c>
-      <x:c r="E3" s="4" t="s">
-        <x:v>500</x:v>
-      </x:c>
-      <x:c r="F3" s="4" t="s">
-        <x:v>534</x:v>
       </x:c>
       <x:c r="G3" s="4" t="s">
         <x:v>159</x:v>
       </x:c>
       <x:c r="H3" s="4" t="s">
-        <x:v>532</x:v>
+        <x:v>531</x:v>
       </x:c>
       <x:c r="I3" s="49">
         <x:v>46277.0</x:v>
@@ -23498,28 +24284,28 @@
     </x:row>
     <x:row r="4">
       <x:c r="A4" s="4" t="s">
-        <x:v>529</x:v>
+        <x:v>528</x:v>
       </x:c>
       <x:c r="B4" s="4" t="s">
-        <x:v>535</x:v>
+        <x:v>534</x:v>
       </x:c>
       <x:c r="C4" s="4" t="s">
         <x:v>162</x:v>
       </x:c>
       <x:c r="D4" s="4" t="s">
+        <x:v>535</x:v>
+      </x:c>
+      <x:c r="E4" s="4" t="s">
         <x:v>536</x:v>
       </x:c>
-      <x:c r="E4" s="4" t="s">
+      <x:c r="F4" s="4" t="s">
         <x:v>537</x:v>
-      </x:c>
-      <x:c r="F4" s="4" t="s">
-        <x:v>538</x:v>
       </x:c>
       <x:c r="G4" s="4" t="s">
         <x:v>166</x:v>
       </x:c>
       <x:c r="H4" s="4" t="s">
-        <x:v>539</x:v>
+        <x:v>538</x:v>
       </x:c>
       <x:c r="I4" s="49">
         <x:v>46277.0</x:v>
@@ -23527,28 +24313,28 @@
     </x:row>
     <x:row r="5">
       <x:c r="A5" s="4" t="s">
+        <x:v>539</x:v>
+      </x:c>
+      <x:c r="B5" s="4" t="s">
         <x:v>540</x:v>
       </x:c>
-      <x:c r="B5" s="4" t="s">
+      <x:c r="C5" s="4" t="s">
         <x:v>541</x:v>
       </x:c>
-      <x:c r="C5" s="4" t="s">
+      <x:c r="D5" s="4" t="s">
         <x:v>542</x:v>
       </x:c>
-      <x:c r="D5" s="4" t="s">
+      <x:c r="E5" s="4" t="s">
         <x:v>543</x:v>
       </x:c>
-      <x:c r="E5" s="4" t="s">
+      <x:c r="F5" s="4" t="s">
         <x:v>544</x:v>
-      </x:c>
-      <x:c r="F5" s="4" t="s">
-        <x:v>545</x:v>
       </x:c>
       <x:c r="G5" s="4" t="s">
         <x:v>173</x:v>
       </x:c>
       <x:c r="H5" s="4" t="s">
-        <x:v>532</x:v>
+        <x:v>531</x:v>
       </x:c>
       <x:c r="I5" s="49">
         <x:v>46277.0</x:v>
@@ -23556,28 +24342,28 @@
     </x:row>
     <x:row r="6">
       <x:c r="A6" s="4" t="s">
+        <x:v>545</x:v>
+      </x:c>
+      <x:c r="B6" s="4" t="s">
         <x:v>546</x:v>
       </x:c>
-      <x:c r="B6" s="4" t="s">
+      <x:c r="C6" s="4" t="s">
+        <x:v>517</x:v>
+      </x:c>
+      <x:c r="D6" s="4" t="s">
         <x:v>547</x:v>
       </x:c>
-      <x:c r="C6" s="4" t="s">
-        <x:v>518</x:v>
-      </x:c>
-      <x:c r="D6" s="4" t="s">
+      <x:c r="E6" s="4" t="s">
         <x:v>548</x:v>
       </x:c>
-      <x:c r="E6" s="4" t="s">
+      <x:c r="F6" s="4" t="s">
         <x:v>549</x:v>
       </x:c>
-      <x:c r="F6" s="4" t="s">
+      <x:c r="G6" s="4" t="s">
         <x:v>550</x:v>
       </x:c>
-      <x:c r="G6" s="4" t="s">
-        <x:v>551</x:v>
-      </x:c>
       <x:c r="H6" s="4" t="s">
-        <x:v>532</x:v>
+        <x:v>531</x:v>
       </x:c>
       <x:c r="I6" s="49">
         <x:v>46277.0</x:v>
@@ -23585,28 +24371,28 @@
     </x:row>
     <x:row r="7">
       <x:c r="A7" s="4" t="s">
-        <x:v>546</x:v>
+        <x:v>545</x:v>
       </x:c>
       <x:c r="B7" s="4" t="s">
-        <x:v>552</x:v>
+        <x:v>551</x:v>
       </x:c>
       <x:c r="C7" s="4" t="s">
         <x:v>142</x:v>
       </x:c>
       <x:c r="D7" s="4" t="s">
+        <x:v>547</x:v>
+      </x:c>
+      <x:c r="E7" s="4" t="s">
         <x:v>548</x:v>
       </x:c>
-      <x:c r="E7" s="4" t="s">
-        <x:v>549</x:v>
-      </x:c>
       <x:c r="F7" s="4" t="s">
+        <x:v>552</x:v>
+      </x:c>
+      <x:c r="G7" s="4" t="s">
         <x:v>553</x:v>
       </x:c>
-      <x:c r="G7" s="4" t="s">
-        <x:v>554</x:v>
-      </x:c>
       <x:c r="H7" s="4" t="s">
-        <x:v>532</x:v>
+        <x:v>531</x:v>
       </x:c>
       <x:c r="I7" s="49">
         <x:v>46277.0</x:v>
@@ -23614,28 +24400,28 @@
     </x:row>
     <x:row r="8">
       <x:c r="A8" s="4" t="s">
-        <x:v>546</x:v>
+        <x:v>545</x:v>
       </x:c>
       <x:c r="B8" s="4" t="s">
-        <x:v>555</x:v>
+        <x:v>554</x:v>
       </x:c>
       <x:c r="C8" s="4" t="s">
         <x:v>162</x:v>
       </x:c>
       <x:c r="D8" s="4" t="s">
+        <x:v>547</x:v>
+      </x:c>
+      <x:c r="E8" s="4" t="s">
         <x:v>548</x:v>
       </x:c>
-      <x:c r="E8" s="4" t="s">
-        <x:v>549</x:v>
-      </x:c>
       <x:c r="F8" s="4" t="s">
+        <x:v>555</x:v>
+      </x:c>
+      <x:c r="G8" s="4" t="s">
         <x:v>556</x:v>
       </x:c>
-      <x:c r="G8" s="4" t="s">
-        <x:v>557</x:v>
-      </x:c>
       <x:c r="H8" s="4" t="s">
-        <x:v>532</x:v>
+        <x:v>531</x:v>
       </x:c>
       <x:c r="I8" s="49">
         <x:v>46277.0</x:v>
@@ -23643,28 +24429,28 @@
     </x:row>
     <x:row r="9">
       <x:c r="A9" s="4" t="s">
-        <x:v>546</x:v>
+        <x:v>545</x:v>
       </x:c>
       <x:c r="B9" s="4" t="s">
+        <x:v>557</x:v>
+      </x:c>
+      <x:c r="C9" s="4" t="s">
         <x:v>558</x:v>
       </x:c>
-      <x:c r="C9" s="4" t="s">
+      <x:c r="D9" s="4" t="s">
         <x:v>559</x:v>
       </x:c>
-      <x:c r="D9" s="4" t="s">
+      <x:c r="E9" s="4" t="s">
+        <x:v>548</x:v>
+      </x:c>
+      <x:c r="F9" s="4" t="s">
         <x:v>560</x:v>
       </x:c>
-      <x:c r="E9" s="4" t="s">
-        <x:v>549</x:v>
-      </x:c>
-      <x:c r="F9" s="4" t="s">
+      <x:c r="G9" s="4" t="s">
         <x:v>561</x:v>
       </x:c>
-      <x:c r="G9" s="4" t="s">
-        <x:v>562</x:v>
-      </x:c>
       <x:c r="H9" s="4" t="s">
-        <x:v>532</x:v>
+        <x:v>531</x:v>
       </x:c>
       <x:c r="I9" s="49">
         <x:v>46277.0</x:v>
@@ -23672,28 +24458,28 @@
     </x:row>
     <x:row r="10">
       <x:c r="A10" s="4" t="s">
-        <x:v>546</x:v>
+        <x:v>545</x:v>
       </x:c>
       <x:c r="B10" s="4" t="s">
+        <x:v>562</x:v>
+      </x:c>
+      <x:c r="C10" s="4" t="s">
         <x:v>563</x:v>
       </x:c>
-      <x:c r="C10" s="4" t="s">
+      <x:c r="D10" s="4" t="s">
         <x:v>564</x:v>
       </x:c>
-      <x:c r="D10" s="4" t="s">
+      <x:c r="E10" s="4" t="s">
+        <x:v>548</x:v>
+      </x:c>
+      <x:c r="F10" s="4" t="s">
         <x:v>565</x:v>
       </x:c>
-      <x:c r="E10" s="4" t="s">
-        <x:v>549</x:v>
-      </x:c>
-      <x:c r="F10" s="4" t="s">
+      <x:c r="G10" s="4" t="s">
         <x:v>566</x:v>
       </x:c>
-      <x:c r="G10" s="4" t="s">
-        <x:v>567</x:v>
-      </x:c>
       <x:c r="H10" s="4" t="s">
-        <x:v>532</x:v>
+        <x:v>531</x:v>
       </x:c>
       <x:c r="I10" s="49">
         <x:v>46277.0</x:v>
@@ -23701,28 +24487,28 @@
     </x:row>
     <x:row r="11">
       <x:c r="A11" s="4" t="s">
+        <x:v>567</x:v>
+      </x:c>
+      <x:c r="B11" s="4" t="s">
         <x:v>568</x:v>
       </x:c>
-      <x:c r="B11" s="4" t="s">
+      <x:c r="C11" s="4" t="s">
         <x:v>569</x:v>
       </x:c>
-      <x:c r="C11" s="4" t="s">
+      <x:c r="D11" s="4" t="s">
+        <x:v>547</x:v>
+      </x:c>
+      <x:c r="E11" s="4" t="s">
+        <x:v>548</x:v>
+      </x:c>
+      <x:c r="F11" s="4" t="s">
         <x:v>570</x:v>
       </x:c>
-      <x:c r="D11" s="4" t="s">
-        <x:v>548</x:v>
-      </x:c>
-      <x:c r="E11" s="4" t="s">
-        <x:v>549</x:v>
-      </x:c>
-      <x:c r="F11" s="4" t="s">
+      <x:c r="G11" s="4" t="s">
         <x:v>571</x:v>
       </x:c>
-      <x:c r="G11" s="4" t="s">
+      <x:c r="H11" s="4" t="s">
         <x:v>572</x:v>
-      </x:c>
-      <x:c r="H11" s="4" t="s">
-        <x:v>573</x:v>
       </x:c>
       <x:c r="I11" s="49">
         <x:v>46277.0</x:v>
@@ -23730,28 +24516,28 @@
     </x:row>
     <x:row r="12">
       <x:c r="A12" s="4" t="s">
-        <x:v>568</x:v>
+        <x:v>567</x:v>
       </x:c>
       <x:c r="B12" s="4" t="s">
+        <x:v>573</x:v>
+      </x:c>
+      <x:c r="C12" s="4" t="s">
         <x:v>574</x:v>
       </x:c>
-      <x:c r="C12" s="4" t="s">
+      <x:c r="D12" s="4" t="s">
+        <x:v>547</x:v>
+      </x:c>
+      <x:c r="E12" s="4" t="s">
+        <x:v>548</x:v>
+      </x:c>
+      <x:c r="F12" s="4" t="s">
         <x:v>575</x:v>
       </x:c>
-      <x:c r="D12" s="4" t="s">
-        <x:v>548</x:v>
-      </x:c>
-      <x:c r="E12" s="4" t="s">
-        <x:v>549</x:v>
-      </x:c>
-      <x:c r="F12" s="4" t="s">
+      <x:c r="G12" s="4" t="s">
         <x:v>576</x:v>
       </x:c>
-      <x:c r="G12" s="4" t="s">
-        <x:v>577</x:v>
-      </x:c>
       <x:c r="H12" s="4" t="s">
-        <x:v>573</x:v>
+        <x:v>572</x:v>
       </x:c>
       <x:c r="I12" s="49">
         <x:v>46277.0</x:v>
@@ -23759,28 +24545,28 @@
     </x:row>
     <x:row r="13">
       <x:c r="A13" s="4" t="s">
-        <x:v>568</x:v>
+        <x:v>567</x:v>
       </x:c>
       <x:c r="B13" s="4" t="s">
+        <x:v>577</x:v>
+      </x:c>
+      <x:c r="C13" s="4" t="s">
+        <x:v>577</x:v>
+      </x:c>
+      <x:c r="D13" s="4" t="s">
+        <x:v>547</x:v>
+      </x:c>
+      <x:c r="E13" s="4" t="s">
+        <x:v>548</x:v>
+      </x:c>
+      <x:c r="F13" s="4" t="s">
         <x:v>578</x:v>
       </x:c>
-      <x:c r="C13" s="4" t="s">
-        <x:v>578</x:v>
-      </x:c>
-      <x:c r="D13" s="4" t="s">
-        <x:v>548</x:v>
-      </x:c>
-      <x:c r="E13" s="4" t="s">
-        <x:v>549</x:v>
-      </x:c>
-      <x:c r="F13" s="4" t="s">
+      <x:c r="G13" s="4" t="s">
         <x:v>579</x:v>
       </x:c>
-      <x:c r="G13" s="4" t="s">
-        <x:v>580</x:v>
-      </x:c>
       <x:c r="H13" s="4" t="s">
-        <x:v>573</x:v>
+        <x:v>572</x:v>
       </x:c>
       <x:c r="I13" s="49">
         <x:v>46277.0</x:v>
@@ -23788,28 +24574,28 @@
     </x:row>
     <x:row r="14">
       <x:c r="A14" s="4" t="s">
-        <x:v>568</x:v>
+        <x:v>567</x:v>
       </x:c>
       <x:c r="B14" s="4" t="s">
+        <x:v>580</x:v>
+      </x:c>
+      <x:c r="C14" s="4" t="s">
+        <x:v>580</x:v>
+      </x:c>
+      <x:c r="D14" s="4" t="s">
+        <x:v>547</x:v>
+      </x:c>
+      <x:c r="E14" s="4" t="s">
+        <x:v>548</x:v>
+      </x:c>
+      <x:c r="F14" s="4" t="s">
         <x:v>581</x:v>
       </x:c>
-      <x:c r="C14" s="4" t="s">
-        <x:v>581</x:v>
-      </x:c>
-      <x:c r="D14" s="4" t="s">
-        <x:v>548</x:v>
-      </x:c>
-      <x:c r="E14" s="4" t="s">
-        <x:v>549</x:v>
-      </x:c>
-      <x:c r="F14" s="4" t="s">
+      <x:c r="G14" s="4" t="s">
         <x:v>582</x:v>
       </x:c>
-      <x:c r="G14" s="4" t="s">
-        <x:v>583</x:v>
-      </x:c>
       <x:c r="H14" s="4" t="s">
-        <x:v>532</x:v>
+        <x:v>531</x:v>
       </x:c>
       <x:c r="I14" s="49">
         <x:v>46277.0</x:v>
@@ -23817,28 +24603,28 @@
     </x:row>
     <x:row r="15">
       <x:c r="A15" s="4" t="s">
-        <x:v>568</x:v>
+        <x:v>567</x:v>
       </x:c>
       <x:c r="B15" s="4" t="s">
+        <x:v>583</x:v>
+      </x:c>
+      <x:c r="C15" s="4" t="s">
+        <x:v>583</x:v>
+      </x:c>
+      <x:c r="D15" s="4" t="s">
+        <x:v>547</x:v>
+      </x:c>
+      <x:c r="E15" s="4" t="s">
+        <x:v>548</x:v>
+      </x:c>
+      <x:c r="F15" s="4" t="s">
         <x:v>584</x:v>
       </x:c>
-      <x:c r="C15" s="4" t="s">
-        <x:v>584</x:v>
-      </x:c>
-      <x:c r="D15" s="4" t="s">
-        <x:v>548</x:v>
-      </x:c>
-      <x:c r="E15" s="4" t="s">
-        <x:v>549</x:v>
-      </x:c>
-      <x:c r="F15" s="4" t="s">
+      <x:c r="G15" s="4" t="s">
         <x:v>585</x:v>
       </x:c>
-      <x:c r="G15" s="4" t="s">
-        <x:v>586</x:v>
-      </x:c>
       <x:c r="H15" s="4" t="s">
-        <x:v>573</x:v>
+        <x:v>572</x:v>
       </x:c>
       <x:c r="I15" s="49">
         <x:v>46277.0</x:v>
@@ -23846,28 +24632,28 @@
     </x:row>
     <x:row r="16">
       <x:c r="A16" s="4" t="s">
-        <x:v>568</x:v>
+        <x:v>567</x:v>
       </x:c>
       <x:c r="B16" s="4" t="s">
+        <x:v>586</x:v>
+      </x:c>
+      <x:c r="C16" s="4" t="s">
+        <x:v>586</x:v>
+      </x:c>
+      <x:c r="D16" s="4" t="s">
+        <x:v>547</x:v>
+      </x:c>
+      <x:c r="E16" s="4" t="s">
+        <x:v>517</x:v>
+      </x:c>
+      <x:c r="F16" s="4" t="s">
         <x:v>587</x:v>
       </x:c>
-      <x:c r="C16" s="4" t="s">
-        <x:v>587</x:v>
-      </x:c>
-      <x:c r="D16" s="4" t="s">
-        <x:v>548</x:v>
-      </x:c>
-      <x:c r="E16" s="4" t="s">
-        <x:v>518</x:v>
-      </x:c>
-      <x:c r="F16" s="4" t="s">
+      <x:c r="G16" s="4" t="s">
         <x:v>588</x:v>
       </x:c>
-      <x:c r="G16" s="4" t="s">
-        <x:v>589</x:v>
-      </x:c>
       <x:c r="H16" s="4" t="s">
-        <x:v>573</x:v>
+        <x:v>572</x:v>
       </x:c>
       <x:c r="I16" s="49">
         <x:v>46277.0</x:v>
@@ -23875,28 +24661,28 @@
     </x:row>
     <x:row r="17">
       <x:c r="A17" s="4" t="s">
-        <x:v>568</x:v>
+        <x:v>567</x:v>
       </x:c>
       <x:c r="B17" s="4" t="s">
+        <x:v>589</x:v>
+      </x:c>
+      <x:c r="C17" s="4" t="s">
         <x:v>590</x:v>
       </x:c>
-      <x:c r="C17" s="4" t="s">
+      <x:c r="D17" s="4" t="s">
+        <x:v>559</x:v>
+      </x:c>
+      <x:c r="E17" s="4" t="s">
+        <x:v>548</x:v>
+      </x:c>
+      <x:c r="F17" s="4" t="s">
         <x:v>591</x:v>
       </x:c>
-      <x:c r="D17" s="4" t="s">
-        <x:v>560</x:v>
-      </x:c>
-      <x:c r="E17" s="4" t="s">
-        <x:v>549</x:v>
-      </x:c>
-      <x:c r="F17" s="4" t="s">
+      <x:c r="G17" s="4" t="s">
         <x:v>592</x:v>
       </x:c>
-      <x:c r="G17" s="4" t="s">
-        <x:v>593</x:v>
-      </x:c>
       <x:c r="H17" s="4" t="s">
-        <x:v>532</x:v>
+        <x:v>531</x:v>
       </x:c>
       <x:c r="I17" s="49">
         <x:v>46277.0</x:v>
@@ -23904,28 +24690,28 @@
     </x:row>
     <x:row r="18">
       <x:c r="A18" s="4" t="s">
-        <x:v>568</x:v>
+        <x:v>567</x:v>
       </x:c>
       <x:c r="B18" s="4" t="s">
+        <x:v>593</x:v>
+      </x:c>
+      <x:c r="C18" s="4" t="s">
+        <x:v>593</x:v>
+      </x:c>
+      <x:c r="D18" s="4" t="s">
+        <x:v>564</x:v>
+      </x:c>
+      <x:c r="E18" s="4" t="s">
+        <x:v>548</x:v>
+      </x:c>
+      <x:c r="F18" s="4" t="s">
         <x:v>594</x:v>
       </x:c>
-      <x:c r="C18" s="4" t="s">
-        <x:v>594</x:v>
-      </x:c>
-      <x:c r="D18" s="4" t="s">
-        <x:v>565</x:v>
-      </x:c>
-      <x:c r="E18" s="4" t="s">
-        <x:v>549</x:v>
-      </x:c>
-      <x:c r="F18" s="4" t="s">
+      <x:c r="G18" s="4" t="s">
         <x:v>595</x:v>
       </x:c>
-      <x:c r="G18" s="4" t="s">
-        <x:v>596</x:v>
-      </x:c>
       <x:c r="H18" s="4" t="s">
-        <x:v>532</x:v>
+        <x:v>531</x:v>
       </x:c>
       <x:c r="I18" s="49">
         <x:v>46277.0</x:v>
@@ -23933,28 +24719,28 @@
     </x:row>
     <x:row r="19">
       <x:c r="A19" s="4" t="s">
+        <x:v>596</x:v>
+      </x:c>
+      <x:c r="B19" s="4" t="s">
         <x:v>597</x:v>
-      </x:c>
-      <x:c r="B19" s="4" t="s">
-        <x:v>598</x:v>
       </x:c>
       <x:c r="C19" s="4" t="s">
         <x:v>189</x:v>
       </x:c>
       <x:c r="D19" s="4" t="s">
+        <x:v>547</x:v>
+      </x:c>
+      <x:c r="E19" s="4" t="s">
         <x:v>548</x:v>
       </x:c>
-      <x:c r="E19" s="4" t="s">
-        <x:v>549</x:v>
-      </x:c>
       <x:c r="F19" s="4" t="s">
-        <x:v>599</x:v>
+        <x:v>598</x:v>
       </x:c>
       <x:c r="G19" s="4" t="s">
         <x:v>193</x:v>
       </x:c>
       <x:c r="H19" s="4" t="s">
-        <x:v>532</x:v>
+        <x:v>531</x:v>
       </x:c>
       <x:c r="I19" s="49">
         <x:v>46277.0</x:v>
@@ -23962,28 +24748,28 @@
     </x:row>
     <x:row r="20">
       <x:c r="A20" s="4" t="s">
-        <x:v>597</x:v>
+        <x:v>596</x:v>
       </x:c>
       <x:c r="B20" s="4" t="s">
+        <x:v>599</x:v>
+      </x:c>
+      <x:c r="C20" s="4" t="s">
+        <x:v>599</x:v>
+      </x:c>
+      <x:c r="D20" s="4" t="s">
+        <x:v>547</x:v>
+      </x:c>
+      <x:c r="E20" s="4" t="s">
+        <x:v>548</x:v>
+      </x:c>
+      <x:c r="F20" s="4" t="s">
         <x:v>600</x:v>
       </x:c>
-      <x:c r="C20" s="4" t="s">
-        <x:v>600</x:v>
-      </x:c>
-      <x:c r="D20" s="4" t="s">
-        <x:v>548</x:v>
-      </x:c>
-      <x:c r="E20" s="4" t="s">
-        <x:v>549</x:v>
-      </x:c>
-      <x:c r="F20" s="4" t="s">
+      <x:c r="G20" s="4" t="s">
         <x:v>601</x:v>
       </x:c>
-      <x:c r="G20" s="4" t="s">
-        <x:v>602</x:v>
-      </x:c>
       <x:c r="H20" s="4" t="s">
-        <x:v>532</x:v>
+        <x:v>531</x:v>
       </x:c>
       <x:c r="I20" s="49">
         <x:v>46277.0</x:v>
@@ -23991,28 +24777,28 @@
     </x:row>
     <x:row r="21" ht="15.75" customHeight="1">
       <x:c r="A21" s="4" t="s">
-        <x:v>597</x:v>
+        <x:v>596</x:v>
       </x:c>
       <x:c r="B21" s="4" t="s">
+        <x:v>602</x:v>
+      </x:c>
+      <x:c r="C21" s="4" t="s">
+        <x:v>602</x:v>
+      </x:c>
+      <x:c r="D21" s="4" t="s">
+        <x:v>547</x:v>
+      </x:c>
+      <x:c r="E21" s="4" t="s">
+        <x:v>548</x:v>
+      </x:c>
+      <x:c r="F21" s="4" t="s">
         <x:v>603</x:v>
       </x:c>
-      <x:c r="C21" s="4" t="s">
-        <x:v>603</x:v>
-      </x:c>
-      <x:c r="D21" s="4" t="s">
-        <x:v>548</x:v>
-      </x:c>
-      <x:c r="E21" s="4" t="s">
-        <x:v>549</x:v>
-      </x:c>
-      <x:c r="F21" s="4" t="s">
+      <x:c r="G21" s="4" t="s">
         <x:v>604</x:v>
       </x:c>
-      <x:c r="G21" s="4" t="s">
-        <x:v>605</x:v>
-      </x:c>
       <x:c r="H21" s="4" t="s">
-        <x:v>573</x:v>
+        <x:v>572</x:v>
       </x:c>
       <x:c r="I21" s="49">
         <x:v>46277.0</x:v>
@@ -24020,28 +24806,28 @@
     </x:row>
     <x:row r="22" ht="15.75" customHeight="1">
       <x:c r="A22" s="4" t="s">
-        <x:v>597</x:v>
+        <x:v>596</x:v>
       </x:c>
       <x:c r="B22" s="4" t="s">
+        <x:v>605</x:v>
+      </x:c>
+      <x:c r="C22" s="4" t="s">
+        <x:v>605</x:v>
+      </x:c>
+      <x:c r="D22" s="4" t="s">
+        <x:v>547</x:v>
+      </x:c>
+      <x:c r="E22" s="4" t="s">
+        <x:v>548</x:v>
+      </x:c>
+      <x:c r="F22" s="4" t="s">
         <x:v>606</x:v>
       </x:c>
-      <x:c r="C22" s="4" t="s">
-        <x:v>606</x:v>
-      </x:c>
-      <x:c r="D22" s="4" t="s">
-        <x:v>548</x:v>
-      </x:c>
-      <x:c r="E22" s="4" t="s">
-        <x:v>549</x:v>
-      </x:c>
-      <x:c r="F22" s="4" t="s">
+      <x:c r="G22" s="4" t="s">
         <x:v>607</x:v>
       </x:c>
-      <x:c r="G22" s="4" t="s">
-        <x:v>608</x:v>
-      </x:c>
       <x:c r="H22" s="4" t="s">
-        <x:v>573</x:v>
+        <x:v>572</x:v>
       </x:c>
       <x:c r="I22" s="49">
         <x:v>46277.0</x:v>
@@ -24049,28 +24835,28 @@
     </x:row>
     <x:row r="23" ht="15.75" customHeight="1">
       <x:c r="A23" s="4" t="s">
-        <x:v>597</x:v>
+        <x:v>596</x:v>
       </x:c>
       <x:c r="B23" s="4" t="s">
+        <x:v>608</x:v>
+      </x:c>
+      <x:c r="C23" s="4" t="s">
+        <x:v>608</x:v>
+      </x:c>
+      <x:c r="D23" s="4" t="s">
+        <x:v>559</x:v>
+      </x:c>
+      <x:c r="E23" s="4" t="s">
+        <x:v>548</x:v>
+      </x:c>
+      <x:c r="F23" s="4" t="s">
         <x:v>609</x:v>
       </x:c>
-      <x:c r="C23" s="4" t="s">
-        <x:v>609</x:v>
-      </x:c>
-      <x:c r="D23" s="4" t="s">
-        <x:v>560</x:v>
-      </x:c>
-      <x:c r="E23" s="4" t="s">
-        <x:v>549</x:v>
-      </x:c>
-      <x:c r="F23" s="4" t="s">
+      <x:c r="G23" s="4" t="s">
         <x:v>610</x:v>
       </x:c>
-      <x:c r="G23" s="4" t="s">
-        <x:v>611</x:v>
-      </x:c>
       <x:c r="H23" s="4" t="s">
-        <x:v>532</x:v>
+        <x:v>531</x:v>
       </x:c>
       <x:c r="I23" s="49">
         <x:v>46277.0</x:v>
@@ -24078,28 +24864,28 @@
     </x:row>
     <x:row r="24" ht="15.75" customHeight="1">
       <x:c r="A24" s="4" t="s">
-        <x:v>597</x:v>
+        <x:v>596</x:v>
       </x:c>
       <x:c r="B24" s="4" t="s">
+        <x:v>611</x:v>
+      </x:c>
+      <x:c r="C24" s="4" t="s">
+        <x:v>611</x:v>
+      </x:c>
+      <x:c r="D24" s="4" t="s">
+        <x:v>564</x:v>
+      </x:c>
+      <x:c r="E24" s="4" t="s">
+        <x:v>548</x:v>
+      </x:c>
+      <x:c r="F24" s="4" t="s">
         <x:v>612</x:v>
       </x:c>
-      <x:c r="C24" s="4" t="s">
-        <x:v>612</x:v>
-      </x:c>
-      <x:c r="D24" s="4" t="s">
-        <x:v>565</x:v>
-      </x:c>
-      <x:c r="E24" s="4" t="s">
-        <x:v>549</x:v>
-      </x:c>
-      <x:c r="F24" s="4" t="s">
+      <x:c r="G24" s="4" t="s">
         <x:v>613</x:v>
       </x:c>
-      <x:c r="G24" s="4" t="s">
-        <x:v>614</x:v>
-      </x:c>
       <x:c r="H24" s="4" t="s">
-        <x:v>532</x:v>
+        <x:v>531</x:v>
       </x:c>
       <x:c r="I24" s="49">
         <x:v>46277.0</x:v>
@@ -24107,7 +24893,7 @@
     </x:row>
     <x:row r="25" ht="15.75" customHeight="1">
       <x:c r="A25" s="4" t="s">
-        <x:v>615</x:v>
+        <x:v>614</x:v>
       </x:c>
       <x:c r="B25" s="4" t="s">
         <x:v>197</x:v>
@@ -24116,19 +24902,19 @@
         <x:v>197</x:v>
       </x:c>
       <x:c r="D25" s="4" t="s">
+        <x:v>547</x:v>
+      </x:c>
+      <x:c r="E25" s="4" t="s">
         <x:v>548</x:v>
       </x:c>
-      <x:c r="E25" s="4" t="s">
-        <x:v>549</x:v>
-      </x:c>
       <x:c r="F25" s="4" t="s">
-        <x:v>616</x:v>
+        <x:v>615</x:v>
       </x:c>
       <x:c r="G25" s="4" t="s">
         <x:v>201</x:v>
       </x:c>
       <x:c r="H25" s="4" t="s">
-        <x:v>532</x:v>
+        <x:v>531</x:v>
       </x:c>
       <x:c r="I25" s="49">
         <x:v>46277.0</x:v>
@@ -24136,28 +24922,28 @@
     </x:row>
     <x:row r="26" ht="15.75" customHeight="1">
       <x:c r="A26" s="4" t="s">
-        <x:v>615</x:v>
+        <x:v>614</x:v>
       </x:c>
       <x:c r="B26" s="4" t="s">
+        <x:v>616</x:v>
+      </x:c>
+      <x:c r="C26" s="4" t="s">
         <x:v>617</x:v>
       </x:c>
-      <x:c r="C26" s="4" t="s">
+      <x:c r="D26" s="4" t="s">
+        <x:v>547</x:v>
+      </x:c>
+      <x:c r="E26" s="4" t="s">
+        <x:v>548</x:v>
+      </x:c>
+      <x:c r="F26" s="4" t="s">
         <x:v>618</x:v>
       </x:c>
-      <x:c r="D26" s="4" t="s">
-        <x:v>548</x:v>
-      </x:c>
-      <x:c r="E26" s="4" t="s">
-        <x:v>549</x:v>
-      </x:c>
-      <x:c r="F26" s="4" t="s">
+      <x:c r="G26" s="4" t="s">
         <x:v>619</x:v>
       </x:c>
-      <x:c r="G26" s="4" t="s">
-        <x:v>620</x:v>
-      </x:c>
       <x:c r="H26" s="4" t="s">
-        <x:v>532</x:v>
+        <x:v>531</x:v>
       </x:c>
       <x:c r="I26" s="49">
         <x:v>46277.0</x:v>
@@ -24165,28 +24951,28 @@
     </x:row>
     <x:row r="27" ht="15.75" customHeight="1">
       <x:c r="A27" s="4" t="s">
-        <x:v>615</x:v>
+        <x:v>614</x:v>
       </x:c>
       <x:c r="B27" s="4" t="s">
+        <x:v>620</x:v>
+      </x:c>
+      <x:c r="C27" s="4" t="s">
+        <x:v>517</x:v>
+      </x:c>
+      <x:c r="D27" s="4" t="s">
+        <x:v>559</x:v>
+      </x:c>
+      <x:c r="E27" s="4" t="s">
+        <x:v>548</x:v>
+      </x:c>
+      <x:c r="F27" s="4" t="s">
         <x:v>621</x:v>
       </x:c>
-      <x:c r="C27" s="4" t="s">
-        <x:v>518</x:v>
-      </x:c>
-      <x:c r="D27" s="4" t="s">
-        <x:v>560</x:v>
-      </x:c>
-      <x:c r="E27" s="4" t="s">
-        <x:v>549</x:v>
-      </x:c>
-      <x:c r="F27" s="4" t="s">
+      <x:c r="G27" s="4" t="s">
         <x:v>622</x:v>
       </x:c>
-      <x:c r="G27" s="4" t="s">
-        <x:v>623</x:v>
-      </x:c>
       <x:c r="H27" s="4" t="s">
-        <x:v>532</x:v>
+        <x:v>531</x:v>
       </x:c>
       <x:c r="I27" s="49">
         <x:v>46277.0</x:v>
@@ -24194,28 +24980,28 @@
     </x:row>
     <x:row r="28" ht="15.75" customHeight="1">
       <x:c r="A28" s="4" t="s">
-        <x:v>615</x:v>
+        <x:v>614</x:v>
       </x:c>
       <x:c r="B28" s="4" t="s">
-        <x:v>624</x:v>
+        <x:v>623</x:v>
       </x:c>
       <x:c r="C28" s="4" t="s">
         <x:v>142</x:v>
       </x:c>
       <x:c r="D28" s="4" t="s">
-        <x:v>565</x:v>
+        <x:v>564</x:v>
       </x:c>
       <x:c r="E28" s="4" t="s">
-        <x:v>549</x:v>
+        <x:v>548</x:v>
       </x:c>
       <x:c r="F28" s="4" t="s">
+        <x:v>624</x:v>
+      </x:c>
+      <x:c r="G28" s="4" t="s">
         <x:v>625</x:v>
       </x:c>
-      <x:c r="G28" s="4" t="s">
-        <x:v>626</x:v>
-      </x:c>
       <x:c r="H28" s="4" t="s">
-        <x:v>532</x:v>
+        <x:v>531</x:v>
       </x:c>
       <x:c r="I28" s="49">
         <x:v>46277.0</x:v>
@@ -24223,28 +25009,28 @@
     </x:row>
     <x:row r="29" ht="15.75" customHeight="1">
       <x:c r="A29" s="4" t="s">
+        <x:v>626</x:v>
+      </x:c>
+      <x:c r="B29" s="4" t="s">
         <x:v>627</x:v>
-      </x:c>
-      <x:c r="B29" s="4" t="s">
-        <x:v>628</x:v>
       </x:c>
       <x:c r="C29" s="4" t="s">
         <x:v>97</x:v>
       </x:c>
       <x:c r="D29" s="4" t="s">
+        <x:v>547</x:v>
+      </x:c>
+      <x:c r="E29" s="4" t="s">
         <x:v>548</x:v>
       </x:c>
-      <x:c r="E29" s="4" t="s">
-        <x:v>549</x:v>
-      </x:c>
       <x:c r="F29" s="4" t="s">
-        <x:v>629</x:v>
+        <x:v>628</x:v>
       </x:c>
       <x:c r="G29" s="4" t="s">
         <x:v>131</x:v>
       </x:c>
       <x:c r="H29" s="4" t="s">
-        <x:v>532</x:v>
+        <x:v>531</x:v>
       </x:c>
       <x:c r="I29" s="49">
         <x:v>46277.0</x:v>
@@ -24252,28 +25038,28 @@
     </x:row>
     <x:row r="30" ht="15.75" customHeight="1">
       <x:c r="A30" s="4" t="s">
-        <x:v>627</x:v>
+        <x:v>626</x:v>
       </x:c>
       <x:c r="B30" s="4" t="s">
-        <x:v>630</x:v>
+        <x:v>629</x:v>
       </x:c>
       <x:c r="C30" s="4" t="s">
         <x:v>176</x:v>
       </x:c>
       <x:c r="D30" s="4" t="s">
-        <x:v>560</x:v>
+        <x:v>559</x:v>
       </x:c>
       <x:c r="E30" s="4" t="s">
-        <x:v>549</x:v>
+        <x:v>548</x:v>
       </x:c>
       <x:c r="F30" s="4" t="s">
-        <x:v>631</x:v>
+        <x:v>630</x:v>
       </x:c>
       <x:c r="G30" s="4" t="s">
         <x:v>180</x:v>
       </x:c>
       <x:c r="H30" s="4" t="s">
-        <x:v>532</x:v>
+        <x:v>531</x:v>
       </x:c>
       <x:c r="I30" s="49">
         <x:v>46277.0</x:v>
@@ -24281,28 +25067,28 @@
     </x:row>
     <x:row r="31" ht="15.75" customHeight="1">
       <x:c r="A31" s="4" t="s">
-        <x:v>627</x:v>
+        <x:v>626</x:v>
       </x:c>
       <x:c r="B31" s="4" t="s">
-        <x:v>632</x:v>
+        <x:v>631</x:v>
       </x:c>
       <x:c r="C31" s="4" t="s">
         <x:v>176</x:v>
       </x:c>
       <x:c r="D31" s="4" t="s">
-        <x:v>565</x:v>
+        <x:v>564</x:v>
       </x:c>
       <x:c r="E31" s="4" t="s">
-        <x:v>549</x:v>
+        <x:v>548</x:v>
       </x:c>
       <x:c r="F31" s="4" t="s">
-        <x:v>633</x:v>
+        <x:v>632</x:v>
       </x:c>
       <x:c r="G31" s="4" t="s">
         <x:v>186</x:v>
       </x:c>
       <x:c r="H31" s="4" t="s">
-        <x:v>532</x:v>
+        <x:v>531</x:v>
       </x:c>
       <x:c r="I31" s="49">
         <x:v>46277.0</x:v>
@@ -25988,28 +26774,28 @@
   <x:sheetData>
     <x:row r="1" ht="33.75" customHeight="1">
       <x:c r="A1" s="34" t="s">
-        <x:v>396</x:v>
+        <x:v>395</x:v>
       </x:c>
       <x:c r="B1" s="34" t="s">
         <x:v>353</x:v>
       </x:c>
       <x:c r="C1" s="34" t="s">
-        <x:v>634</x:v>
+        <x:v>633</x:v>
       </x:c>
       <x:c r="D1" s="34" t="s">
         <x:v>65</x:v>
       </x:c>
       <x:c r="E1" s="34" t="s">
+        <x:v>634</x:v>
+      </x:c>
+      <x:c r="F1" s="34" t="s">
         <x:v>635</x:v>
       </x:c>
-      <x:c r="F1" s="34" t="s">
+      <x:c r="G1" s="34" t="s">
         <x:v>636</x:v>
       </x:c>
-      <x:c r="G1" s="34" t="s">
+      <x:c r="H1" s="34" t="s">
         <x:v>637</x:v>
-      </x:c>
-      <x:c r="H1" s="34" t="s">
-        <x:v>638</x:v>
       </x:c>
     </x:row>
     <x:row r="2">
@@ -26020,22 +26806,22 @@
         <x:v>9</x:v>
       </x:c>
       <x:c r="C2" s="4" t="s">
+        <x:v>638</x:v>
+      </x:c>
+      <x:c r="D2" s="4" t="s">
         <x:v>639</x:v>
       </x:c>
-      <x:c r="D2" s="4" t="s">
+      <x:c r="E2" s="4" t="s">
         <x:v>640</x:v>
       </x:c>
-      <x:c r="E2" s="4" t="s">
+      <x:c r="F2" s="4" t="s">
         <x:v>641</x:v>
-      </x:c>
-      <x:c r="F2" s="4" t="s">
-        <x:v>642</x:v>
       </x:c>
       <x:c r="G2" s="4" t="s">
         <x:v>113</x:v>
       </x:c>
       <x:c r="H2" s="4" t="s">
-        <x:v>643</x:v>
+        <x:v>642</x:v>
       </x:c>
     </x:row>
     <x:row r="3">
@@ -26046,22 +26832,22 @@
         <x:v>9</x:v>
       </x:c>
       <x:c r="C3" s="4" t="s">
+        <x:v>643</x:v>
+      </x:c>
+      <x:c r="D3" s="4" t="s">
         <x:v>644</x:v>
       </x:c>
-      <x:c r="D3" s="4" t="s">
+      <x:c r="E3" s="4" t="s">
         <x:v>645</x:v>
       </x:c>
-      <x:c r="E3" s="4" t="s">
+      <x:c r="F3" s="4" t="s">
         <x:v>646</x:v>
-      </x:c>
-      <x:c r="F3" s="4" t="s">
-        <x:v>647</x:v>
       </x:c>
       <x:c r="G3" s="4" t="s">
         <x:v>103</x:v>
       </x:c>
       <x:c r="H3" s="4" t="s">
-        <x:v>648</x:v>
+        <x:v>647</x:v>
       </x:c>
     </x:row>
     <x:row r="4">
@@ -26072,22 +26858,22 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="C4" s="4" t="s">
+        <x:v>648</x:v>
+      </x:c>
+      <x:c r="D4" s="4" t="s">
         <x:v>649</x:v>
       </x:c>
-      <x:c r="D4" s="4" t="s">
+      <x:c r="E4" s="4" t="s">
         <x:v>650</x:v>
       </x:c>
-      <x:c r="E4" s="4" t="s">
+      <x:c r="F4" s="4" t="s">
         <x:v>651</x:v>
-      </x:c>
-      <x:c r="F4" s="4" t="s">
-        <x:v>652</x:v>
       </x:c>
       <x:c r="G4" s="4" t="s">
         <x:v>113</x:v>
       </x:c>
       <x:c r="H4" s="4" t="s">
-        <x:v>653</x:v>
+        <x:v>652</x:v>
       </x:c>
     </x:row>
     <x:row r="5">
@@ -26098,22 +26884,22 @@
         <x:v>9</x:v>
       </x:c>
       <x:c r="C5" s="4" t="s">
+        <x:v>653</x:v>
+      </x:c>
+      <x:c r="D5" s="4" t="s">
         <x:v>654</x:v>
       </x:c>
-      <x:c r="D5" s="4" t="s">
+      <x:c r="E5" s="4" t="s">
         <x:v>655</x:v>
       </x:c>
-      <x:c r="E5" s="4" t="s">
+      <x:c r="F5" s="4" t="s">
         <x:v>656</x:v>
-      </x:c>
-      <x:c r="F5" s="4" t="s">
-        <x:v>657</x:v>
       </x:c>
       <x:c r="G5" s="4" t="s">
         <x:v>103</x:v>
       </x:c>
       <x:c r="H5" s="4" t="s">
-        <x:v>658</x:v>
+        <x:v>657</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
@@ -26124,22 +26910,22 @@
         <x:v>13</x:v>
       </x:c>
       <x:c r="C6" s="4" t="s">
+        <x:v>658</x:v>
+      </x:c>
+      <x:c r="D6" s="4" t="s">
         <x:v>659</x:v>
       </x:c>
-      <x:c r="D6" s="4" t="s">
+      <x:c r="E6" s="4" t="s">
         <x:v>660</x:v>
       </x:c>
-      <x:c r="E6" s="4" t="s">
+      <x:c r="F6" s="4" t="s">
         <x:v>661</x:v>
-      </x:c>
-      <x:c r="F6" s="4" t="s">
-        <x:v>662</x:v>
       </x:c>
       <x:c r="G6" s="4" t="s">
         <x:v>113</x:v>
       </x:c>
       <x:c r="H6" s="4" t="s">
-        <x:v>663</x:v>
+        <x:v>662</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
@@ -28056,15 +28842,12 @@
         <x:v>Cobertura</x:v>
       </x:c>
       <x:c r="B5" s="65" t="n">
-        <x:f>COUNTA('Matriz de precios'!A2:A100)</x:f>
-        <x:v>28</x:v>
+        <x:v>40</x:v>
       </x:c>
       <x:c r="C5" s="65" t="n">
-        <x:f>COUNT('Matriz de precios'!G2:G100)</x:f>
-        <x:v>20</x:v>
+        <x:v>32</x:v>
       </x:c>
       <x:c r="D5" s="65" t="n">
-        <x:f>COUNTA('Matriz de precios'!A2:A100)-COUNT('Matriz de precios'!G2:G100)</x:f>
         <x:v>8</x:v>
       </x:c>
       <x:c r="E5" s="66" t="n">
@@ -28077,7 +28860,7 @@
         <x:v>En curso</x:v>
       </x:c>
       <x:c r="H5" s="65" t="str">
-        <x:v>FP-178/FP-182 integradas; FP-166 puede auditar y FP-180/FP-183 pueden consumir</x:v>
+        <x:v>FP-182/FP-183 integradas; 12 categorías Azure por región con fuente oficial</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
@@ -28753,19 +29536,19 @@
         <x:v>46280</x:v>
       </x:c>
       <x:c r="B36" s="65" t="str">
-        <x:v>1.1</x:v>
+        <x:v>1.2</x:v>
       </x:c>
       <x:c r="C36" s="65" t="str">
-        <x:v>FP-126</x:v>
+        <x:v>FP-126 / FP-183</x:v>
       </x:c>
       <x:c r="D36" s="65" t="str">
-        <x:v>Se reemplazó la fila genérica por planes/productos trazables y se agregó control de dependencias.</x:v>
+        <x:v>Se agregaron seis categorías Azure por región y se actualizaron precios de la línea base TCO.</x:v>
       </x:c>
       <x:c r="E36" s="65" t="str">
-        <x:v>Fuentes oficiales enlazadas en la matriz</x:v>
+        <x:v>Azure Retail Prices API</x:v>
       </x:c>
       <x:c r="F36" s="65" t="str">
-        <x:v>FP-180, FP-183, FP-185 y derivados</x:v>
+        <x:v>FP-183, FP-185 y derivados</x:v>
       </x:c>
       <x:c r="G36" s="65" t="str">
         <x:v>Pendiente FP-166</x:v>

</xml_diff>